<commit_message>
feat: update FHIR conversion specification documents with IG update v1.8.1 #2992 - updated global-script
</commit_message>
<xml_diff>
--- a/support/specifications/ccda/CCDA to FHIR Conversion Spec - AthenaHealth.xlsx
+++ b/support/specifications/ccda/CCDA to FHIR Conversion Spec - AthenaHealth.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="28800" windowHeight="12180" tabRatio="709" activeTab="5"/>
+    <workbookView windowWidth="19200" windowHeight="8000" tabRatio="709" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="AthenaHealth" sheetId="11" r:id="rId1"/>
@@ -104,11 +104,23 @@
     <t>"meta" : {
     "lastUpdated" : "2024-02-23T00:00:00Z",
     "profile" : ["http://shinny.org/us/ny/hrsn/StructureDefinition/SHINNYBundleProfile"],
-    "security": [ {
-                  "code": "ETH",
-                  "system": "http://terminology.hl7.org/CodeSystem/v3-ActCode",
-                  "display": "Substance abuse information sensitivity"
-              } ]
+   "security": [
+      {
+        "code": "ETH",
+        "system": "http://terminology.hl7.org/CodeSystem/v3-ActCode",
+        "display": "Substance abuse information sensitivity"
+      },
+      {
+        "code": "MH",
+        "system": "http://terminology.hl7.org/CodeSystem/v3-ActCode",
+        "display": "Mental health information sensitivity"
+      },
+      {
+        "code": "DVD",
+        "system": "http://terminology.hl7.org/CodeSystem/v3-ActCode",
+        "display": "Developmental disability information sensitivity"
+      }
+    ],
   },</t>
   </si>
   <si>
@@ -122,13 +134,6 @@
   </si>
   <si>
     <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF00B050"/>
-        <rFont val="Calibri"/>
-        <charset val="134"/>
-        <scheme val="minor"/>
-      </rPr>
       <t>If the header variable `</t>
     </r>
     <r>
@@ -171,7 +176,51 @@
         <charset val="134"/>
         <scheme val="minor"/>
       </rPr>
-      <t>', then only the meta -&gt; security will be added.</t>
+      <t>', then the 'ETH' code will be added to meta -&gt; security.
+If the header variable `</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF00B050"/>
+        <rFont val="Calibri"/>
+        <charset val="134"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>X-TechBD-OPWDD</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF00B050"/>
+        <rFont val="Calibri"/>
+        <charset val="134"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>` has the value 'True', then the 'DVD' code will be added to meta -&gt; security.
+If the header variable `</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF00B050"/>
+        <rFont val="Calibri"/>
+        <charset val="134"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>X-TechBD-OMH</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF00B050"/>
+        <rFont val="Calibri"/>
+        <charset val="134"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>` has the value 'True', then the 'MH' code will be added to meta -&gt; security.</t>
     </r>
   </si>
   <si>
@@ -635,7 +684,7 @@
 WP, DIR, PUB -&gt; work
 TMP -&gt; temp
 BAD -&gt; old
-All Others (H, HP, HV, AS, EC, MC, PG) -&gt; home</t>
+H, HP, HV -&gt; home</t>
     </r>
   </si>
   <si>
@@ -2649,7 +2698,7 @@
       </rPr>
       <t xml:space="preserve">
 completed -&gt; finished
-norma -&gt; finished 
+normal -&gt; finished 
 active -&gt; in-progress 
 cancelled -&gt; cancelled
 aborted -&gt; cancelled 
@@ -6022,7 +6071,6 @@
     <font>
       <b/>
       <sz val="11"/>
-      <color rgb="FFFF0000"/>
       <name val="Calibri"/>
       <charset val="134"/>
       <scheme val="minor"/>
@@ -6031,6 +6079,14 @@
       <b/>
       <sz val="11"/>
       <color rgb="FFC00000"/>
+      <name val="Calibri"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FFFF0000"/>
       <name val="Calibri"/>
       <charset val="134"/>
       <scheme val="minor"/>
@@ -6068,13 +6124,6 @@
       <color rgb="FF00B050"/>
       <name val="Segoe UI"/>
       <charset val="134"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <name val="Calibri"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="35">
@@ -7182,11 +7231,11 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
   <dimension ref="A1:C7"/>
-  <sheetFormatPr defaultColWidth="8.88571428571429" defaultRowHeight="15" outlineLevelRow="6" outlineLevelCol="2"/>
+  <sheetFormatPr defaultColWidth="8.88181818181818" defaultRowHeight="14.5" outlineLevelRow="6" outlineLevelCol="2"/>
   <cols>
-    <col min="1" max="1" width="8.88571428571429" style="32"/>
-    <col min="2" max="2" width="35.2190476190476" customWidth="1"/>
-    <col min="3" max="3" width="92.6666666666667" customWidth="1"/>
+    <col min="1" max="1" width="8.88181818181818" style="32"/>
+    <col min="2" max="2" width="35.2181818181818" customWidth="1"/>
+    <col min="3" max="3" width="92.6636363636364" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3">
@@ -7259,14 +7308,14 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
   <dimension ref="A1:G17"/>
-  <sheetFormatPr defaultColWidth="9.14285714285714" defaultRowHeight="15" outlineLevelCol="6"/>
+  <sheetFormatPr defaultColWidth="9.14545454545454" defaultRowHeight="14.5" outlineLevelCol="6"/>
   <cols>
-    <col min="1" max="1" width="14.7142857142857" customWidth="1"/>
-    <col min="2" max="2" width="30.8571428571429" customWidth="1"/>
-    <col min="3" max="3" width="63.4285714285714" customWidth="1"/>
-    <col min="4" max="4" width="70.7142857142857" customWidth="1"/>
-    <col min="5" max="5" width="52.4285714285714" customWidth="1"/>
-    <col min="6" max="6" width="57.5714285714286" customWidth="1"/>
+    <col min="1" max="1" width="14.7181818181818" customWidth="1"/>
+    <col min="2" max="2" width="30.8545454545455" customWidth="1"/>
+    <col min="3" max="3" width="63.4272727272727" customWidth="1"/>
+    <col min="4" max="4" width="70.7181818181818" customWidth="1"/>
+    <col min="5" max="5" width="52.4272727272727" customWidth="1"/>
+    <col min="6" max="6" width="57.5727272727273" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" s="1" customFormat="1" spans="1:7">
@@ -7308,7 +7357,7 @@
         <v>431</v>
       </c>
     </row>
-    <row r="4" ht="60" spans="1:7">
+    <row r="4" ht="58" spans="1:7">
       <c r="B4" s="5" t="s">
         <v>16</v>
       </c>
@@ -7330,7 +7379,7 @@
       </c>
       <c r="E5" s="8"/>
     </row>
-    <row r="6" ht="30" spans="1:7">
+    <row r="6" ht="29" spans="1:7">
       <c r="B6" s="5" t="s">
         <v>22</v>
       </c>
@@ -7357,7 +7406,7 @@
       <c r="E7" s="11"/>
       <c r="F7" s="4"/>
     </row>
-    <row r="8" customFormat="1" ht="75" spans="1:7">
+    <row r="8" customFormat="1" ht="72.5" spans="1:7">
       <c r="B8" s="4" t="s">
         <v>84</v>
       </c>
@@ -7371,7 +7420,7 @@
         <v>439</v>
       </c>
     </row>
-    <row r="9" customFormat="1" ht="60" spans="1:7">
+    <row r="9" customFormat="1" ht="58" spans="1:7">
       <c r="B9" s="4" t="s">
         <v>88</v>
       </c>
@@ -7480,14 +7529,14 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
   <dimension ref="A1:F22"/>
-  <sheetFormatPr defaultColWidth="9.14285714285714" defaultRowHeight="15" outlineLevelCol="5"/>
+  <sheetFormatPr defaultColWidth="9.14545454545454" defaultRowHeight="14.5" outlineLevelCol="5"/>
   <cols>
-    <col min="1" max="1" width="14.7142857142857" customWidth="1"/>
-    <col min="2" max="2" width="28.3333333333333" customWidth="1"/>
-    <col min="3" max="3" width="65.6666666666667" customWidth="1"/>
-    <col min="4" max="4" width="46.2190476190476" customWidth="1"/>
-    <col min="5" max="5" width="61.2857142857143" customWidth="1"/>
-    <col min="6" max="6" width="46.2857142857143" customWidth="1"/>
+    <col min="1" max="1" width="14.7181818181818" customWidth="1"/>
+    <col min="2" max="2" width="28.3363636363636" customWidth="1"/>
+    <col min="3" max="3" width="65.6636363636364" customWidth="1"/>
+    <col min="4" max="4" width="46.2181818181818" customWidth="1"/>
+    <col min="5" max="5" width="61.2818181818182" customWidth="1"/>
+    <col min="6" max="6" width="46.2818181818182" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" s="1" customFormat="1" spans="1:6">
@@ -7558,7 +7607,7 @@
       </c>
       <c r="D6" s="29"/>
     </row>
-    <row r="7" s="27" customFormat="1" ht="86" customHeight="1" spans="1:6">
+    <row r="7" s="27" customFormat="1" ht="316" customHeight="1" spans="1:6">
       <c r="A7" s="28"/>
       <c r="B7" s="28" t="s">
         <v>24</v>
@@ -7585,7 +7634,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="10" customFormat="1" ht="30" spans="1:6">
+    <row r="10" customFormat="1" ht="29" spans="1:6">
       <c r="B10" t="s">
         <v>30</v>
       </c>
@@ -7606,7 +7655,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="16" ht="75" spans="1:6">
+    <row r="16" ht="72.5" spans="1:6">
       <c r="B16" t="s">
         <v>35</v>
       </c>
@@ -7622,7 +7671,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="18" ht="75" spans="2:5">
+    <row r="18" ht="72.5" spans="2:5">
       <c r="B18" t="s">
         <v>39</v>
       </c>
@@ -7633,7 +7682,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="19" ht="45" spans="2:5">
+    <row r="19" ht="29" spans="2:5">
       <c r="B19" s="4" t="s">
         <v>42</v>
       </c>
@@ -7642,7 +7691,7 @@
       </c>
       <c r="E19" s="10"/>
     </row>
-    <row r="20" ht="45" spans="2:5">
+    <row r="20" ht="43.5" spans="2:5">
       <c r="B20" t="s">
         <v>44</v>
       </c>
@@ -7651,13 +7700,13 @@
       </c>
       <c r="E20" s="10"/>
     </row>
-    <row r="21" ht="30" spans="2:5">
+    <row r="21" ht="29" spans="2:5">
       <c r="B21" s="4" t="s">
         <v>46</v>
       </c>
       <c r="E21" s="8"/>
     </row>
-    <row r="22" ht="105" spans="2:5">
+    <row r="22" ht="101.5" spans="2:5">
       <c r="B22" s="31" t="s">
         <v>47</v>
       </c>
@@ -7681,13 +7730,13 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
   <dimension ref="A1:F68"/>
-  <sheetFormatPr defaultColWidth="8.88571428571429" defaultRowHeight="15" outlineLevelCol="5"/>
+  <sheetFormatPr defaultColWidth="8.88181818181818" defaultRowHeight="14.5" outlineLevelCol="5"/>
   <cols>
-    <col min="1" max="1" width="14.7142857142857" customWidth="1"/>
-    <col min="2" max="2" width="41.7809523809524" style="4" customWidth="1"/>
-    <col min="3" max="3" width="63.8857142857143" style="4" customWidth="1"/>
-    <col min="4" max="4" width="81.2857142857143" style="4" customWidth="1"/>
-    <col min="5" max="5" width="48.4285714285714" style="4" customWidth="1"/>
+    <col min="1" max="1" width="14.7181818181818" customWidth="1"/>
+    <col min="2" max="2" width="41.7818181818182" style="4" customWidth="1"/>
+    <col min="3" max="3" width="63.8818181818182" style="4" customWidth="1"/>
+    <col min="4" max="4" width="81.2818181818182" style="4" customWidth="1"/>
+    <col min="5" max="5" width="48.4272727272727" style="4" customWidth="1"/>
     <col min="6" max="6" width="45" customWidth="1"/>
   </cols>
   <sheetData>
@@ -7753,7 +7802,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="7" ht="30" spans="1:6">
+    <row r="7" ht="29" spans="1:6">
       <c r="B7" s="4" t="s">
         <v>55</v>
       </c>
@@ -7764,7 +7813,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="8" ht="60" spans="1:6">
+    <row r="8" ht="58" spans="1:6">
       <c r="B8" s="4" t="s">
         <v>58</v>
       </c>
@@ -7820,7 +7869,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="13" ht="60" spans="1:6">
+    <row r="13" ht="58" spans="1:6">
       <c r="B13" s="4" t="s">
         <v>72</v>
       </c>
@@ -7831,7 +7880,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="14" ht="30" spans="1:6">
+    <row r="14" ht="29" spans="1:6">
       <c r="B14" s="4" t="s">
         <v>75</v>
       </c>
@@ -7842,7 +7891,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="15" ht="30" spans="1:6">
+    <row r="15" ht="29" spans="1:6">
       <c r="B15" s="4" t="s">
         <v>78</v>
       </c>
@@ -7864,7 +7913,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="17" ht="75" spans="2:5">
+    <row r="17" ht="72.5" spans="2:5">
       <c r="B17" s="4" t="s">
         <v>84</v>
       </c>
@@ -7878,7 +7927,7 @@
         <v>87</v>
       </c>
     </row>
-    <row r="18" ht="60" spans="2:5">
+    <row r="18" ht="58" spans="2:5">
       <c r="B18" s="4" t="s">
         <v>88</v>
       </c>
@@ -7932,7 +7981,7 @@
       </c>
       <c r="D23" s="12"/>
     </row>
-    <row r="24" ht="120" spans="2:5">
+    <row r="24" ht="116" spans="2:5">
       <c r="B24" s="4" t="s">
         <v>100</v>
       </c>
@@ -7951,7 +8000,7 @@
         <v>104</v>
       </c>
     </row>
-    <row r="26" ht="90" spans="2:5">
+    <row r="26" ht="87" spans="2:5">
       <c r="B26" s="4" t="s">
         <v>105</v>
       </c>
@@ -7962,7 +8011,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="27" ht="45" spans="2:5">
+    <row r="27" ht="43.5" spans="2:5">
       <c r="B27" s="4" t="s">
         <v>108</v>
       </c>
@@ -7976,7 +8025,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="28" ht="30" spans="2:5">
+    <row r="28" spans="2:5">
       <c r="B28" s="4" t="s">
         <v>112</v>
       </c>
@@ -7996,7 +8045,7 @@
       <c r="D29" s="14"/>
       <c r="E29" s="8"/>
     </row>
-    <row r="30" ht="30" spans="2:5">
+    <row r="30" spans="2:5">
       <c r="B30" s="4" t="s">
         <v>116</v>
       </c>
@@ -8016,7 +8065,7 @@
       <c r="D31" s="14"/>
       <c r="E31" s="8"/>
     </row>
-    <row r="32" ht="45" spans="2:5">
+    <row r="32" ht="43.5" spans="2:5">
       <c r="B32" s="4" t="s">
         <v>108</v>
       </c>
@@ -8030,7 +8079,7 @@
         <v>121</v>
       </c>
     </row>
-    <row r="33" ht="30" spans="2:6">
+    <row r="33" spans="2:6">
       <c r="B33" s="4" t="s">
         <v>112</v>
       </c>
@@ -8048,7 +8097,7 @@
       </c>
       <c r="D34" s="14"/>
     </row>
-    <row r="35" ht="30" spans="2:6">
+    <row r="35" spans="2:6">
       <c r="B35" s="4" t="s">
         <v>116</v>
       </c>
@@ -8077,7 +8126,7 @@
         <v>127</v>
       </c>
     </row>
-    <row r="38" ht="45" spans="2:6">
+    <row r="38" ht="43.5" spans="2:6">
       <c r="B38" s="4" t="s">
         <v>128</v>
       </c>
@@ -8089,7 +8138,7 @@
         <v>129</v>
       </c>
     </row>
-    <row r="39" ht="120" spans="2:6">
+    <row r="39" ht="116" spans="2:6">
       <c r="B39" s="4" t="s">
         <v>130</v>
       </c>
@@ -8100,7 +8149,7 @@
         <v>132</v>
       </c>
     </row>
-    <row r="40" ht="120" spans="2:6">
+    <row r="40" ht="116" spans="2:6">
       <c r="B40" s="4" t="s">
         <v>133</v>
       </c>
@@ -8147,7 +8196,7 @@
       </c>
       <c r="D44" s="10"/>
     </row>
-    <row r="45" ht="195" spans="2:6">
+    <row r="45" ht="188.5" spans="2:6">
       <c r="B45" s="15" t="s">
         <v>143</v>
       </c>
@@ -8161,7 +8210,7 @@
         <v>146</v>
       </c>
     </row>
-    <row r="46" ht="195" spans="2:6">
+    <row r="46" ht="188.5" spans="2:6">
       <c r="B46" s="15" t="s">
         <v>147</v>
       </c>
@@ -8175,7 +8224,7 @@
         <v>150</v>
       </c>
     </row>
-    <row r="47" ht="195" spans="2:6">
+    <row r="47" ht="188.5" spans="2:6">
       <c r="B47" s="15" t="s">
         <v>151</v>
       </c>
@@ -8227,7 +8276,7 @@
       <c r="D51" s="10"/>
       <c r="E51" s="4"/>
     </row>
-    <row r="52" ht="150" spans="2:6">
+    <row r="52" ht="145" spans="2:6">
       <c r="B52" s="10" t="s">
         <v>160</v>
       </c>
@@ -8301,7 +8350,7 @@
       <c r="D58" s="10"/>
       <c r="E58" s="8"/>
     </row>
-    <row r="59" ht="180" spans="2:6">
+    <row r="59" ht="174" spans="2:6">
       <c r="B59" s="10" t="s">
         <v>174</v>
       </c>
@@ -8315,7 +8364,7 @@
         <v>176</v>
       </c>
     </row>
-    <row r="60" ht="255" spans="2:6">
+    <row r="60" ht="246.5" spans="2:6">
       <c r="B60" s="4" t="s">
         <v>177</v>
       </c>
@@ -8346,7 +8395,7 @@
       <c r="D62" s="10"/>
       <c r="F62" s="4"/>
     </row>
-    <row r="63" ht="210" spans="2:6">
+    <row r="63" ht="203" spans="2:6">
       <c r="B63" s="4" t="s">
         <v>184</v>
       </c>
@@ -8424,14 +8473,14 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
   <dimension ref="A1:G22"/>
-  <sheetFormatPr defaultColWidth="9.14285714285714" defaultRowHeight="15" outlineLevelCol="6"/>
+  <sheetFormatPr defaultColWidth="9.14545454545454" defaultRowHeight="14.5" outlineLevelCol="6"/>
   <cols>
-    <col min="1" max="1" width="14.7142857142857" customWidth="1"/>
-    <col min="2" max="2" width="30.8571428571429" customWidth="1"/>
-    <col min="3" max="3" width="63.4285714285714" customWidth="1"/>
-    <col min="4" max="4" width="70.7142857142857" customWidth="1"/>
-    <col min="5" max="5" width="52.4285714285714" customWidth="1"/>
-    <col min="6" max="6" width="57.5714285714286" customWidth="1"/>
+    <col min="1" max="1" width="14.7181818181818" customWidth="1"/>
+    <col min="2" max="2" width="30.8545454545455" customWidth="1"/>
+    <col min="3" max="3" width="63.4272727272727" customWidth="1"/>
+    <col min="4" max="4" width="70.7181818181818" customWidth="1"/>
+    <col min="5" max="5" width="52.4272727272727" customWidth="1"/>
+    <col min="6" max="6" width="57.5727272727273" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" s="1" customFormat="1" spans="1:7">
@@ -8473,7 +8522,7 @@
         <v>198</v>
       </c>
     </row>
-    <row r="4" ht="60" spans="1:7">
+    <row r="4" ht="58" spans="1:7">
       <c r="B4" s="5" t="s">
         <v>16</v>
       </c>
@@ -8504,7 +8553,7 @@
       </c>
       <c r="E6" s="26"/>
     </row>
-    <row r="7" ht="120" spans="1:7">
+    <row r="7" ht="116" spans="1:7">
       <c r="B7" s="5" t="s">
         <v>202</v>
       </c>
@@ -8557,7 +8606,7 @@
         <v>209</v>
       </c>
     </row>
-    <row r="11" ht="225" spans="1:7">
+    <row r="11" ht="203" spans="1:7">
       <c r="B11" s="5" t="s">
         <v>214</v>
       </c>
@@ -8593,7 +8642,7 @@
         <v>209</v>
       </c>
     </row>
-    <row r="14" ht="45" spans="1:7">
+    <row r="14" ht="43.5" spans="1:7">
       <c r="B14" s="5" t="s">
         <v>221</v>
       </c>
@@ -8607,7 +8656,7 @@
         <v>224</v>
       </c>
     </row>
-    <row r="15" ht="255" spans="1:7">
+    <row r="15" ht="246.5" spans="1:7">
       <c r="B15" s="5" t="s">
         <v>225</v>
       </c>
@@ -8621,7 +8670,7 @@
         <v>228</v>
       </c>
     </row>
-    <row r="16" ht="45" spans="1:7">
+    <row r="16" ht="43.5" spans="1:7">
       <c r="B16" s="5" t="s">
         <v>229</v>
       </c>
@@ -8633,7 +8682,7 @@
       </c>
       <c r="E16" s="8"/>
     </row>
-    <row r="17" ht="45" spans="2:6">
+    <row r="17" ht="43.5" spans="2:6">
       <c r="B17" s="5" t="s">
         <v>232</v>
       </c>
@@ -8645,7 +8694,7 @@
       </c>
       <c r="E17" s="8"/>
     </row>
-    <row r="18" ht="45" spans="2:6">
+    <row r="18" ht="43.5" spans="2:6">
       <c r="B18" t="s">
         <v>235</v>
       </c>
@@ -8659,7 +8708,7 @@
         <v>209</v>
       </c>
     </row>
-    <row r="19" ht="60" spans="2:6">
+    <row r="19" ht="58" spans="2:6">
       <c r="B19" s="5" t="s">
         <v>238</v>
       </c>
@@ -8724,14 +8773,14 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
   <dimension ref="A1:F26"/>
-  <sheetFormatPr defaultColWidth="9.14285714285714" defaultRowHeight="15" outlineLevelCol="5"/>
+  <sheetFormatPr defaultColWidth="9.14545454545454" defaultRowHeight="14.5" outlineLevelCol="5"/>
   <cols>
-    <col min="1" max="1" width="14.7142857142857" customWidth="1"/>
-    <col min="2" max="2" width="35.1428571428571" customWidth="1"/>
-    <col min="3" max="3" width="42.2857142857143" style="4" customWidth="1"/>
-    <col min="4" max="4" width="73.5714285714286" customWidth="1"/>
+    <col min="1" max="1" width="14.7181818181818" customWidth="1"/>
+    <col min="2" max="2" width="35.1454545454545" customWidth="1"/>
+    <col min="3" max="3" width="42.2818181818182" style="4" customWidth="1"/>
+    <col min="4" max="4" width="73.5727272727273" customWidth="1"/>
     <col min="5" max="5" width="53" customWidth="1"/>
-    <col min="6" max="6" width="51.7142857142857" customWidth="1"/>
+    <col min="6" max="6" width="51.7181818181818" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" s="1" customFormat="1" spans="1:6">
@@ -8773,7 +8822,7 @@
         <v>246</v>
       </c>
     </row>
-    <row r="4" ht="75" spans="1:6">
+    <row r="4" ht="72.5" spans="1:6">
       <c r="A4" s="1"/>
       <c r="B4" s="5" t="s">
         <v>16</v>
@@ -8800,7 +8849,7 @@
       <c r="E5" s="4"/>
       <c r="F5" s="4"/>
     </row>
-    <row r="6" customFormat="1" ht="30" spans="1:6">
+    <row r="6" customFormat="1" ht="29" spans="1:6">
       <c r="B6" s="15" t="s">
         <v>22</v>
       </c>
@@ -8811,7 +8860,7 @@
       <c r="E6" s="4"/>
       <c r="F6" s="4"/>
     </row>
-    <row r="7" ht="255" spans="1:6">
+    <row r="7" ht="246.5" spans="1:6">
       <c r="B7" s="5" t="s">
         <v>202</v>
       </c>
@@ -8837,7 +8886,7 @@
       </c>
       <c r="E8" s="9"/>
     </row>
-    <row r="9" ht="30" spans="1:6">
+    <row r="9" ht="29" spans="1:6">
       <c r="B9" s="5" t="s">
         <v>256</v>
       </c>
@@ -8857,7 +8906,7 @@
       <c r="D10" s="10"/>
       <c r="E10" s="9"/>
     </row>
-    <row r="11" ht="30" spans="1:6">
+    <row r="11" ht="29" spans="1:6">
       <c r="B11" s="5" t="s">
         <v>260</v>
       </c>
@@ -8868,7 +8917,7 @@
         <v>262</v>
       </c>
     </row>
-    <row r="12" ht="60" spans="1:6">
+    <row r="12" ht="58" spans="1:6">
       <c r="B12" s="5" t="s">
         <v>263</v>
       </c>
@@ -8894,7 +8943,7 @@
         <v>268</v>
       </c>
     </row>
-    <row r="15" customFormat="1" ht="60" spans="1:6">
+    <row r="15" customFormat="1" ht="58" spans="1:6">
       <c r="B15" s="5" t="s">
         <v>269</v>
       </c>
@@ -8905,7 +8954,7 @@
         <v>270</v>
       </c>
     </row>
-    <row r="16" customFormat="1" ht="30" spans="1:6">
+    <row r="16" customFormat="1" ht="29" spans="1:6">
       <c r="B16" s="5" t="s">
         <v>271</v>
       </c>
@@ -8913,7 +8962,7 @@
         <v>272</v>
       </c>
     </row>
-    <row r="17" ht="60" spans="2:5">
+    <row r="17" ht="58" spans="2:5">
       <c r="B17" t="s">
         <v>273</v>
       </c>
@@ -8932,7 +8981,7 @@
         <v>277</v>
       </c>
     </row>
-    <row r="19" ht="45" spans="2:5">
+    <row r="19" ht="43.5" spans="2:5">
       <c r="B19" t="s">
         <v>278</v>
       </c>
@@ -8966,7 +9015,7 @@
         <v>286</v>
       </c>
     </row>
-    <row r="22" ht="60" spans="2:5">
+    <row r="22" ht="58" spans="2:5">
       <c r="B22" t="s">
         <v>287</v>
       </c>
@@ -9035,14 +9084,14 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
   <dimension ref="A1:F32"/>
-  <sheetFormatPr defaultColWidth="9.14285714285714" defaultRowHeight="15" outlineLevelCol="5"/>
+  <sheetFormatPr defaultColWidth="9.14545454545454" defaultRowHeight="14.5" outlineLevelCol="5"/>
   <cols>
-    <col min="1" max="1" width="14.7142857142857" customWidth="1"/>
-    <col min="2" max="2" width="27.3333333333333" customWidth="1"/>
-    <col min="3" max="3" width="50.8857142857143" customWidth="1"/>
-    <col min="4" max="4" width="72.8571428571429" customWidth="1"/>
-    <col min="5" max="5" width="46.4285714285714" customWidth="1"/>
-    <col min="6" max="6" width="45.7142857142857" customWidth="1"/>
+    <col min="1" max="1" width="14.7181818181818" customWidth="1"/>
+    <col min="2" max="2" width="27.3363636363636" customWidth="1"/>
+    <col min="3" max="3" width="50.8818181818182" customWidth="1"/>
+    <col min="4" max="4" width="72.8545454545455" customWidth="1"/>
+    <col min="5" max="5" width="46.4272727272727" customWidth="1"/>
+    <col min="6" max="6" width="45.7181818181818" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" s="1" customFormat="1" spans="1:6">
@@ -9100,7 +9149,7 @@
       </c>
       <c r="F5" s="4"/>
     </row>
-    <row r="6" customFormat="1" ht="30" spans="1:6">
+    <row r="6" customFormat="1" ht="29" spans="1:6">
       <c r="B6" s="4" t="s">
         <v>22</v>
       </c>
@@ -9149,7 +9198,7 @@
       <c r="D9" s="10"/>
       <c r="E9" s="8"/>
     </row>
-    <row r="10" ht="30" spans="1:6">
+    <row r="10" ht="29" spans="1:6">
       <c r="B10" s="4" t="s">
         <v>309</v>
       </c>
@@ -9159,7 +9208,7 @@
       <c r="D10" s="10"/>
       <c r="E10" s="8"/>
     </row>
-    <row r="11" ht="30" spans="1:6">
+    <row r="11" ht="29" spans="1:6">
       <c r="B11" s="4" t="s">
         <v>311</v>
       </c>
@@ -9169,7 +9218,7 @@
       <c r="D11" s="10"/>
       <c r="E11" s="8"/>
     </row>
-    <row r="12" ht="30" spans="1:6">
+    <row r="12" ht="29" spans="1:6">
       <c r="B12" s="4" t="s">
         <v>312</v>
       </c>
@@ -9203,7 +9252,7 @@
       <c r="D14" s="10"/>
       <c r="E14" s="22"/>
     </row>
-    <row r="15" customFormat="1" ht="30" spans="1:6">
+    <row r="15" customFormat="1" ht="29" spans="1:6">
       <c r="B15" s="4" t="s">
         <v>319</v>
       </c>
@@ -9213,7 +9262,7 @@
       <c r="D15" s="10"/>
       <c r="E15" s="22"/>
     </row>
-    <row r="16" customFormat="1" ht="30" spans="1:6">
+    <row r="16" customFormat="1" ht="29" spans="1:6">
       <c r="B16" s="4" t="s">
         <v>321</v>
       </c>
@@ -9223,7 +9272,7 @@
       <c r="D16" s="10"/>
       <c r="E16" s="4"/>
     </row>
-    <row r="17" customFormat="1" ht="30" spans="2:6">
+    <row r="17" customFormat="1" ht="29" spans="2:6">
       <c r="B17" s="4" t="s">
         <v>322</v>
       </c>
@@ -9232,7 +9281,7 @@
       </c>
       <c r="D17" s="10"/>
     </row>
-    <row r="18" ht="30" spans="2:6">
+    <row r="18" ht="29" spans="2:6">
       <c r="B18" s="5" t="s">
         <v>324</v>
       </c>
@@ -9265,7 +9314,7 @@
         <v>331</v>
       </c>
     </row>
-    <row r="21" customFormat="1" ht="120" spans="2:6">
+    <row r="21" customFormat="1" ht="116" spans="2:6">
       <c r="B21" s="4" t="s">
         <v>100</v>
       </c>
@@ -9278,7 +9327,7 @@
       </c>
       <c r="F21" s="4"/>
     </row>
-    <row r="22" customFormat="1" ht="30" spans="2:6">
+    <row r="22" customFormat="1" ht="29" spans="2:6">
       <c r="B22" s="4" t="s">
         <v>103</v>
       </c>
@@ -9288,7 +9337,7 @@
       <c r="D22" s="10"/>
       <c r="F22" s="4"/>
     </row>
-    <row r="23" customFormat="1" ht="90" spans="2:6">
+    <row r="23" customFormat="1" ht="87" spans="2:6">
       <c r="B23" s="4" t="s">
         <v>105</v>
       </c>
@@ -9301,7 +9350,7 @@
       </c>
       <c r="F23" s="4"/>
     </row>
-    <row r="24" customFormat="1" ht="120" spans="2:6">
+    <row r="24" customFormat="1" ht="116" spans="2:6">
       <c r="B24" s="4" t="s">
         <v>88</v>
       </c>
@@ -9314,7 +9363,7 @@
       <c r="E24" s="4"/>
       <c r="F24" s="4"/>
     </row>
-    <row r="25" customFormat="1" ht="75" spans="2:6">
+    <row r="25" customFormat="1" ht="72.5" spans="2:6">
       <c r="B25" s="4" t="s">
         <v>84</v>
       </c>
@@ -9327,7 +9376,7 @@
       </c>
       <c r="F25" s="4"/>
     </row>
-    <row r="26" customFormat="1" ht="30" spans="2:6">
+    <row r="26" customFormat="1" ht="29" spans="2:6">
       <c r="B26" s="4" t="s">
         <v>90</v>
       </c>
@@ -9338,7 +9387,7 @@
       <c r="E26" s="4"/>
       <c r="F26" s="4"/>
     </row>
-    <row r="27" customFormat="1" ht="30" spans="2:6">
+    <row r="27" customFormat="1" ht="29" spans="2:6">
       <c r="B27" s="4" t="s">
         <v>92</v>
       </c>
@@ -9349,7 +9398,7 @@
       <c r="E27" s="4"/>
       <c r="F27" s="4"/>
     </row>
-    <row r="28" customFormat="1" ht="30" spans="2:6">
+    <row r="28" customFormat="1" ht="29" spans="2:6">
       <c r="B28" s="4" t="s">
         <v>94</v>
       </c>
@@ -9360,7 +9409,7 @@
       <c r="E28" s="4"/>
       <c r="F28" s="4"/>
     </row>
-    <row r="29" customFormat="1" ht="30" spans="2:6">
+    <row r="29" customFormat="1" ht="29" spans="2:6">
       <c r="B29" s="4" t="s">
         <v>96</v>
       </c>
@@ -9371,7 +9420,7 @@
       <c r="E29" s="4"/>
       <c r="F29" s="4"/>
     </row>
-    <row r="30" customFormat="1" ht="30" spans="2:6">
+    <row r="30" customFormat="1" ht="29" spans="2:6">
       <c r="B30" s="4" t="s">
         <v>98</v>
       </c>
@@ -9420,13 +9469,13 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
   <dimension ref="A1:F21"/>
-  <sheetFormatPr defaultColWidth="8.88571428571429" defaultRowHeight="15" outlineLevelCol="5"/>
+  <sheetFormatPr defaultColWidth="8.88181818181818" defaultRowHeight="14.5" outlineLevelCol="5"/>
   <cols>
-    <col min="1" max="1" width="14.7142857142857" customWidth="1"/>
-    <col min="2" max="2" width="33.8857142857143" customWidth="1"/>
-    <col min="3" max="3" width="46.8571428571429" customWidth="1"/>
-    <col min="4" max="4" width="57.1142857142857" customWidth="1"/>
-    <col min="5" max="5" width="54.7142857142857" customWidth="1"/>
+    <col min="1" max="1" width="14.7181818181818" customWidth="1"/>
+    <col min="2" max="2" width="33.8818181818182" customWidth="1"/>
+    <col min="3" max="3" width="46.8545454545455" customWidth="1"/>
+    <col min="4" max="4" width="57.1181818181818" customWidth="1"/>
+    <col min="5" max="5" width="54.7181818181818" customWidth="1"/>
     <col min="6" max="6" width="38" customWidth="1"/>
   </cols>
   <sheetData>
@@ -9450,7 +9499,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="2" ht="45" spans="1:6">
+    <row r="2" ht="43.5" spans="1:6">
       <c r="A2" s="21" t="s">
         <v>347</v>
       </c>
@@ -9488,7 +9537,7 @@
       <c r="E5" s="4"/>
       <c r="F5" s="4"/>
     </row>
-    <row r="6" ht="30" spans="1:6">
+    <row r="6" ht="29" spans="1:6">
       <c r="B6" s="15" t="s">
         <v>22</v>
       </c>
@@ -9510,7 +9559,7 @@
         <v>351</v>
       </c>
     </row>
-    <row r="8" ht="150" spans="1:6">
+    <row r="8" ht="145" spans="1:6">
       <c r="B8" s="5" t="s">
         <v>202</v>
       </c>
@@ -9535,7 +9584,7 @@
         <v>357</v>
       </c>
     </row>
-    <row r="10" ht="30" spans="1:6">
+    <row r="10" ht="29" spans="1:6">
       <c r="B10" s="5" t="s">
         <v>358</v>
       </c>
@@ -9554,7 +9603,7 @@
       <c r="D11" s="10"/>
       <c r="E11" s="8"/>
     </row>
-    <row r="12" ht="30" spans="1:6">
+    <row r="12" ht="29" spans="1:6">
       <c r="B12" s="5" t="s">
         <v>361</v>
       </c>
@@ -9574,7 +9623,7 @@
         <v>364</v>
       </c>
     </row>
-    <row r="14" ht="30" spans="1:6">
+    <row r="14" ht="29" spans="1:6">
       <c r="B14" s="4" t="s">
         <v>365</v>
       </c>
@@ -9595,7 +9644,7 @@
         <v>369</v>
       </c>
     </row>
-    <row r="16" ht="75" spans="1:6">
+    <row r="16" ht="58" spans="1:6">
       <c r="B16" s="5" t="s">
         <v>269</v>
       </c>
@@ -9606,7 +9655,7 @@
         <v>270</v>
       </c>
     </row>
-    <row r="17" ht="30" spans="2:6">
+    <row r="17" ht="29" spans="2:6">
       <c r="B17" s="5" t="s">
         <v>271</v>
       </c>
@@ -9614,7 +9663,7 @@
         <v>272</v>
       </c>
     </row>
-    <row r="18" ht="90" spans="2:6">
+    <row r="18" ht="87" spans="2:6">
       <c r="B18" t="s">
         <v>370</v>
       </c>
@@ -9674,14 +9723,14 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
   <dimension ref="A1:F31"/>
-  <sheetFormatPr defaultColWidth="9.14285714285714" defaultRowHeight="15" outlineLevelCol="5"/>
+  <sheetFormatPr defaultColWidth="9.14545454545454" defaultRowHeight="14.5" outlineLevelCol="5"/>
   <cols>
-    <col min="1" max="1" width="14.7142857142857" customWidth="1"/>
-    <col min="2" max="2" width="34.5714285714286" customWidth="1"/>
-    <col min="3" max="3" width="49.6666666666667" customWidth="1"/>
-    <col min="4" max="4" width="56.552380952381" customWidth="1"/>
-    <col min="5" max="5" width="53.2857142857143" customWidth="1"/>
-    <col min="6" max="6" width="50.2857142857143" customWidth="1"/>
+    <col min="1" max="1" width="14.7181818181818" customWidth="1"/>
+    <col min="2" max="2" width="34.5727272727273" customWidth="1"/>
+    <col min="3" max="3" width="49.6636363636364" customWidth="1"/>
+    <col min="4" max="4" width="56.5545454545455" customWidth="1"/>
+    <col min="5" max="5" width="53.2818181818182" customWidth="1"/>
+    <col min="6" max="6" width="50.2818181818182" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" s="1" customFormat="1" spans="1:6">
@@ -9725,7 +9774,7 @@
         <v>348</v>
       </c>
     </row>
-    <row r="4" ht="78" spans="1:6">
+    <row r="4" ht="82.5" spans="1:6">
       <c r="A4" s="1"/>
       <c r="B4" s="5" t="s">
         <v>16</v>
@@ -9750,7 +9799,7 @@
       <c r="E5" s="4"/>
       <c r="F5" s="4"/>
     </row>
-    <row r="6" customFormat="1" ht="30" spans="1:6">
+    <row r="6" customFormat="1" ht="29" spans="1:6">
       <c r="B6" s="15" t="s">
         <v>22</v>
       </c>
@@ -9772,7 +9821,7 @@
         <v>351</v>
       </c>
     </row>
-    <row r="8" ht="105" spans="1:6">
+    <row r="8" ht="101.5" spans="1:6">
       <c r="B8" s="5" t="s">
         <v>202</v>
       </c>
@@ -9797,7 +9846,7 @@
         <v>387</v>
       </c>
     </row>
-    <row r="10" ht="45" spans="1:6">
+    <row r="10" ht="43.5" spans="1:6">
       <c r="B10" s="5" t="s">
         <v>219</v>
       </c>
@@ -9809,7 +9858,7 @@
         <v>389</v>
       </c>
     </row>
-    <row r="11" ht="210" spans="1:6">
+    <row r="11" ht="203" spans="1:6">
       <c r="B11" s="5" t="s">
         <v>214</v>
       </c>
@@ -9818,7 +9867,7 @@
         <v>390</v>
       </c>
     </row>
-    <row r="12" ht="210" spans="1:6">
+    <row r="12" ht="203" spans="1:6">
       <c r="B12" s="5" t="s">
         <v>217</v>
       </c>
@@ -9870,7 +9919,7 @@
       <c r="D16" s="10"/>
       <c r="E16" s="9"/>
     </row>
-    <row r="17" ht="30" spans="2:6">
+    <row r="17" ht="29" spans="2:6">
       <c r="B17" s="5" t="s">
         <v>361</v>
       </c>
@@ -9882,7 +9931,7 @@
         <v>397</v>
       </c>
     </row>
-    <row r="18" ht="105" spans="2:6">
+    <row r="18" ht="101.5" spans="2:6">
       <c r="B18" s="4" t="s">
         <v>362</v>
       </c>
@@ -9896,7 +9945,7 @@
         <v>400</v>
       </c>
     </row>
-    <row r="19" ht="30" spans="2:6">
+    <row r="19" ht="29" spans="2:6">
       <c r="B19" s="4" t="s">
         <v>365</v>
       </c>
@@ -9904,7 +9953,7 @@
         <v>401</v>
       </c>
     </row>
-    <row r="20" ht="30" spans="2:6">
+    <row r="20" ht="29" spans="2:6">
       <c r="B20" s="4" t="s">
         <v>367</v>
       </c>
@@ -9924,7 +9973,7 @@
       </c>
       <c r="E21" s="8"/>
     </row>
-    <row r="22" ht="75" spans="2:6">
+    <row r="22" ht="72.5" spans="2:6">
       <c r="B22" s="5" t="s">
         <v>405</v>
       </c>
@@ -9936,7 +9985,7 @@
         <v>407</v>
       </c>
     </row>
-    <row r="23" ht="45" spans="2:6">
+    <row r="23" ht="43.5" spans="2:6">
       <c r="B23" s="5" t="s">
         <v>408</v>
       </c>
@@ -9945,7 +9994,7 @@
         <v>409</v>
       </c>
     </row>
-    <row r="24" ht="75" spans="2:6">
+    <row r="24" ht="58" spans="2:6">
       <c r="B24" s="5" t="s">
         <v>269</v>
       </c>
@@ -9956,7 +10005,7 @@
         <v>270</v>
       </c>
     </row>
-    <row r="25" ht="30" spans="2:6">
+    <row r="25" ht="29" spans="2:6">
       <c r="B25" s="5" t="s">
         <v>271</v>
       </c>
@@ -9964,7 +10013,7 @@
         <v>272</v>
       </c>
     </row>
-    <row r="26" ht="45" spans="2:6">
+    <row r="26" ht="43.5" spans="2:6">
       <c r="B26" s="5" t="s">
         <v>410</v>
       </c>
@@ -9975,7 +10024,7 @@
         <v>412</v>
       </c>
     </row>
-    <row r="27" ht="210" spans="2:6">
+    <row r="27" ht="203" spans="2:6">
       <c r="B27" s="5" t="s">
         <v>370</v>
       </c>
@@ -9987,7 +10036,7 @@
         <v>413</v>
       </c>
     </row>
-    <row r="28" ht="45" spans="2:6">
+    <row r="28" ht="43.5" spans="2:6">
       <c r="B28" s="5" t="s">
         <v>414</v>
       </c>
@@ -10047,14 +10096,14 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
   <dimension ref="A1:F21"/>
-  <sheetFormatPr defaultColWidth="9.14285714285714" defaultRowHeight="15" outlineLevelCol="5"/>
+  <sheetFormatPr defaultColWidth="9.14545454545454" defaultRowHeight="14.5" outlineLevelCol="5"/>
   <cols>
-    <col min="1" max="1" width="14.7142857142857" customWidth="1"/>
-    <col min="2" max="2" width="33.5714285714286" customWidth="1"/>
-    <col min="3" max="3" width="49.6666666666667" customWidth="1"/>
-    <col min="4" max="4" width="56.552380952381" customWidth="1"/>
-    <col min="5" max="5" width="53.2857142857143" customWidth="1"/>
-    <col min="6" max="6" width="47.5714285714286" customWidth="1"/>
+    <col min="1" max="1" width="14.7181818181818" customWidth="1"/>
+    <col min="2" max="2" width="33.5727272727273" customWidth="1"/>
+    <col min="3" max="3" width="49.6636363636364" customWidth="1"/>
+    <col min="4" max="4" width="56.5545454545455" customWidth="1"/>
+    <col min="5" max="5" width="53.2818181818182" customWidth="1"/>
+    <col min="6" max="6" width="47.5727272727273" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" s="1" customFormat="1" spans="1:6">
@@ -10122,7 +10171,7 @@
       <c r="E5" s="4"/>
       <c r="F5" s="4"/>
     </row>
-    <row r="6" customFormat="1" ht="30" spans="1:6">
+    <row r="6" customFormat="1" ht="29" spans="1:6">
       <c r="B6" s="15" t="s">
         <v>22</v>
       </c>
@@ -10147,7 +10196,7 @@
         <v>351</v>
       </c>
     </row>
-    <row r="8" ht="105" spans="1:6">
+    <row r="8" ht="101.5" spans="1:6">
       <c r="B8" s="5" t="s">
         <v>202</v>
       </c>
@@ -10173,7 +10222,7 @@
         <v>421</v>
       </c>
     </row>
-    <row r="10" ht="165" spans="1:6">
+    <row r="10" ht="159.5" spans="1:6">
       <c r="B10" s="5" t="s">
         <v>355</v>
       </c>
@@ -10187,7 +10236,7 @@
         <v>423</v>
       </c>
     </row>
-    <row r="11" ht="180" spans="1:6">
+    <row r="11" ht="159.5" spans="1:6">
       <c r="B11" s="5" t="s">
         <v>358</v>
       </c>
@@ -10196,7 +10245,7 @@
         <v>424</v>
       </c>
     </row>
-    <row r="12" ht="150" spans="1:6">
+    <row r="12" ht="145" spans="1:6">
       <c r="B12" s="5" t="s">
         <v>360</v>
       </c>
@@ -10205,7 +10254,7 @@
         <v>425</v>
       </c>
     </row>
-    <row r="13" ht="75" spans="1:6">
+    <row r="13" ht="58" spans="1:6">
       <c r="B13" s="5" t="s">
         <v>269</v>
       </c>
@@ -10216,7 +10265,7 @@
         <v>270</v>
       </c>
     </row>
-    <row r="14" ht="30" spans="1:6">
+    <row r="14" ht="29" spans="1:6">
       <c r="B14" s="5" t="s">
         <v>271</v>
       </c>
@@ -10224,7 +10273,7 @@
         <v>272</v>
       </c>
     </row>
-    <row r="15" ht="45" spans="1:6">
+    <row r="15" ht="43.5" spans="1:6">
       <c r="B15" s="5" t="s">
         <v>410</v>
       </c>
@@ -10235,7 +10284,7 @@
         <v>412</v>
       </c>
     </row>
-    <row r="16" ht="210" spans="1:6">
+    <row r="16" ht="203" spans="1:6">
       <c r="B16" s="5" t="s">
         <v>370</v>
       </c>
@@ -10247,7 +10296,7 @@
         <v>413</v>
       </c>
     </row>
-    <row r="17" ht="45" spans="2:6">
+    <row r="17" ht="43.5" spans="2:6">
       <c r="B17" s="5" t="s">
         <v>414</v>
       </c>
@@ -10272,7 +10321,7 @@
         <v>376</v>
       </c>
     </row>
-    <row r="19" ht="165" spans="2:6">
+    <row r="19" ht="159.5" spans="2:6">
       <c r="B19" t="s">
         <v>427</v>
       </c>

</xml_diff>

<commit_message>
docs: update CCDA to FHIR conversion specification documents for Epic, Medent and AthenaHealth with the resource ID generation logic #3080
</commit_message>
<xml_diff>
--- a/support/specifications/ccda/CCDA to FHIR Conversion Spec - AthenaHealth.xlsx
+++ b/support/specifications/ccda/CCDA to FHIR Conversion Spec - AthenaHealth.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="19200" windowHeight="8000" tabRatio="709" activeTab="1"/>
+    <workbookView windowWidth="28800" windowHeight="12180" tabRatio="709" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="AthenaHealth" sheetId="11" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="697" uniqueCount="450">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="697" uniqueCount="456">
   <si>
     <t>AthenaHealth CCDA</t>
   </si>
@@ -89,10 +89,33 @@
     <t>id</t>
   </si>
   <si>
-    <t>Generated dynamically</t>
-  </si>
-  <si>
-    <t>"id" : "AHCHRSNQuestionnaireResponseExample",</t>
+    <r>
+      <t>Randomly generated UUID which is used as the</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF00B050"/>
+        <rFont val="Calibri"/>
+        <charset val="134"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> Interaction ID</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF00B050"/>
+        <rFont val="Calibri"/>
+        <charset val="134"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>.</t>
+    </r>
+  </si>
+  <si>
+    <t>"id" : "041e4b7d-fa8c-41dc-b712-8ed47f3cd0d3",</t>
   </si>
   <si>
     <t>meta -&gt; lastUpdated</t>
@@ -134,6 +157,13 @@
   </si>
   <si>
     <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF00B050"/>
+        <rFont val="Calibri"/>
+        <charset val="134"/>
+        <scheme val="minor"/>
+      </rPr>
       <t>If the header variable `</t>
     </r>
     <r>
@@ -489,7 +519,13 @@
     <t>"Patient"</t>
   </si>
   <si>
-    <t>"id" : "PatientExample",</t>
+    <t>SHA-256 UUID generated using 
+1. Patient-MRN (the value set for 'identifier (MR) -&gt; value' of Patient Resource from Document.recordTarget.patientRole.id.extension)
+2. Value of the header variable 'X-TechBD-CIN'
+3. Content of first occurance of Patient section from Document.recordTarget.patientRole.</t>
+  </si>
+  <si>
+    <t>"id" : "cb71544f4e9980fb01120627d3685a31ed9b0f0f53c6d414c963dcd87df34ae",</t>
   </si>
   <si>
     <t>The bundle generation time.</t>
@@ -1952,7 +1988,11 @@
     <t>"Consent"</t>
   </si>
   <si>
-    <t>Unique 64-character SHA-256 Consent resource ID is generated using the Patient MRN, Patient CIN, current timestamp, and the text content of the resource (if present) in the CCDA XML file.</t>
+    <t>SHA-256 UUID generated using 
+1. Patient-MRN (the value set for 'identifier (MR) -&gt; value' of Patient Resource from Document.recordTarget.patientRole.id.extension)
+2. Value of the header variable 'X-TechBD-CIN'
+3. Content of first occurance of Consent section from Document.authorization.consent
+4. CurrentTimestamp</t>
   </si>
   <si>
     <t>Bundle generation time.</t>
@@ -2602,37 +2642,16 @@
     <t>"Encounter"</t>
   </si>
   <si>
-    <t>"id" : "EncounterExample",</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="Calibri"/>
-        <charset val="134"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>If the encompassingEncounter section is present in the CCDA XML file (</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <rFont val="Calibri"/>
-        <charset val="134"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>AthenaHealth</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="Calibri"/>
-        <charset val="134"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> CCDA files), a 64-character SHA-256 Encounter resource ID is generated from the Patient MRN, Patient CIN, effectiveTime, and the text content of the encompassingEncounter section (if any).</t>
-    </r>
+    <t>SHA-256 UUID generated using 
+1. Patient-MRN (the value set for 'identifier (MR) -&gt; value' of Patient Resource from Document.recordTarget.patientRole.id.extension)
+2. Value of the header variable 'X-TechBD-CIN'
+3. Encounter Effective Time (the value set for 'period -&gt; start' from effectiveTime.low.value)
+4. Content of encounter section
+Document.componentOf.encompassingEncounter OR
+Document.component.structuredBody.component.section[code.code='46240-8'].entry[0].encounter</t>
+  </si>
+  <si>
+    <t>"id" : "90e37429459ebf1f23b950867db2d26c4a8e2cb684b6c2dc3fca3d88ee34725",</t>
   </si>
   <si>
     <t>"http://shinny.org/us/ny/hrsn/StructureDefinition/shinny-encounter"</t>
@@ -3449,6 +3468,15 @@
     <t>"Organization"</t>
   </si>
   <si>
+    <t>SHA-256 UUID generated using 
+1. Patient-MRN (the value set for 'identifier (MR) -&gt; value' of Patient Resource from Document.recordTarget.patientRole.id.extension)
+2. Value of the header variable 'X-TechBD-CIN'
+3. Content of first occurance of Document.author section</t>
+  </si>
+  <si>
+    <t>"id" : "8e4752d52cb9f94657401368f1c8e3cdb052624b10166a665e4c80cdabc62b3c",</t>
+  </si>
+  <si>
     <t>Tentatively mapped the last updated date time.</t>
   </si>
   <si>
@@ -4013,7 +4041,16 @@
     <t>"Observation"</t>
   </si>
   <si>
-    <t>"id" : "S8845918CUMC20250121T1024400530",</t>
+    <t>Facility ID (from the header variable `X-TechBD-Facility-ID`) + '-' + position of the section + '-' +  Value of Document.component.structuredBody.component.section[code.code='29762-2'].entry.observation.id.extension
+If id.extension is not available then will use 
+SHA-256 UUID generated using 
+1. Patient-MRN (the value set for 'identifier (MR) -&gt; value' of Patient Resource from Document.recordTarget.patientRole.id.extension)
+2. Value of the header variable 'X-TechBD-CIN'
+3. Content of the observation section from Document.component.structuredBody.component.section[code.code='29762-2'].entry.observation
+"position of the section" is used to handle multiple sexual orientation resources.</t>
+  </si>
+  <si>
+    <t>"id" : "ACPNY-43Z549669.1",</t>
   </si>
   <si>
     <t>"http://shinny.org/us/ny/hrsn/StructureDefinition/shinny-observation-sexual-orientation"</t>
@@ -4359,137 +4396,11 @@
     </r>
   </si>
   <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF00B050"/>
-        <rFont val="Calibri"/>
-        <charset val="134"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Combine the Facility ID obtained from the header variable '</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="9"/>
-        <color rgb="FF00B050"/>
-        <rFont val="Consolas"/>
-        <charset val="134"/>
-      </rPr>
-      <t xml:space="preserve">X-TechBD-Facility-ID' </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="9"/>
-        <color rgb="FF00B050"/>
-        <rFont val="Consolas"/>
-        <charset val="134"/>
-      </rPr>
-      <t>and</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="9"/>
-        <color rgb="FF00B050"/>
-        <rFont val="Consolas"/>
-        <charset val="134"/>
-      </rPr>
-      <t xml:space="preserve"> </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="10.5"/>
-        <color rgb="FF00B050"/>
-        <rFont val="Segoe UI"/>
-        <charset val="134"/>
-      </rPr>
-      <t>code.code</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="9"/>
-        <color rgb="FF00B050"/>
-        <rFont val="Consolas"/>
-        <charset val="134"/>
-      </rPr>
-      <t xml:space="preserve"> </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10.5"/>
-        <color rgb="FF00B050"/>
-        <rFont val="Segoe UI"/>
-        <charset val="134"/>
-      </rPr>
-      <t>with the</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="10.5"/>
-        <color rgb="FF00B050"/>
-        <rFont val="Segoe UI"/>
-        <charset val="134"/>
-      </rPr>
-      <t xml:space="preserve"> id.extension</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10.5"/>
-        <color rgb="FF00B050"/>
-        <rFont val="Segoe UI"/>
-        <charset val="134"/>
-      </rPr>
-      <t xml:space="preserve"> value from the Observation element.
-If </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="10.5"/>
-        <color rgb="FF00B050"/>
-        <rFont val="Segoe UI"/>
-        <charset val="134"/>
-      </rPr>
-      <t>id.extension</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10.5"/>
-        <color rgb="FF00B050"/>
-        <rFont val="Segoe UI"/>
-        <charset val="134"/>
-      </rPr>
-      <t xml:space="preserve"> is not available then add </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="10.5"/>
-        <color rgb="FF00B050"/>
-        <rFont val="Segoe UI"/>
-        <charset val="134"/>
-      </rPr>
-      <t>effectiveDateTime</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10.5"/>
-        <color rgb="FF00B050"/>
-        <rFont val="Segoe UI"/>
-        <charset val="134"/>
-      </rPr>
-      <t xml:space="preserve"> calculated.</t>
-    </r>
-  </si>
-  <si>
-    <t>"id": "ACPNY-96778-6-20260217000000"
-OR
-"id": "ACPNY-96778-6-flo1570000081-5810220439-97066-Z549669"</t>
+    <t>Facility ID (from the header variable `X-TechBD-Facility-ID`) + '-' + question code (code.code) + '-' + id.extension value from the Observation element.
+If id.extension is not available then will use effectiveDateTime calculated of the observation resource.</t>
+  </si>
+  <si>
+    <t>"id": "ACPNY-88122-7-flo1572879820-5810220439-97051-Z549669"</t>
   </si>
   <si>
     <t>"http://shinny.org/us/ny/hrsn/StructureDefinition/shinny-observation-screening-response"</t>
@@ -5199,7 +5110,17 @@
     </r>
   </si>
   <si>
-    <t>"id" : "N6645918CUMC20250121T1024400530",</t>
+    <t>Facility ID (from the header variable `X-TechBD-Facility-ID`) + '-' + SHA-256 UUID generated using 
+1. Patient-MRN (the value set for 'identifier (MR) -&gt; value' of Patient Resource from Document.recordTarget.patientRole.id.extension)
+2. Value of the header variable 'X-TechBD-CIN'
+3. Grouper ScreeningCode 
+4. effectiveDateTime of the observation resource from 
+'Document.component.structuredBody.component.section[code.code='47519-4'].entry.observation.effectiveTime.low.value' 
+OR effectiveDateTime of the encounter resource from 
+'Document.component.structuredBody.component.section[code.code='46240-8'].entry[0].encounter.effectiveTime.low.value'</t>
+  </si>
+  <si>
+    <t>"id" : "ACPNY-ce2d8db59199c1e63ac0fe2183f2c18ca3cc68c5ff93976bc",</t>
   </si>
   <si>
     <t>Provided the fixed value, "en"</t>
@@ -5724,7 +5645,15 @@
     <t>"Location"</t>
   </si>
   <si>
-    <t>Unique 64-character SHA-256 Location resource ID is generated using the Patient MRN, Patient CIN, current timestamp, and the text content of the resource (if present) in the CCDA XML file.</t>
+    <t>SHA-256 UUID generated using 
+1. Patient-MRN (the value set for 'identifier (MR) -&gt; value' of Patient Resource from Document.recordTarget.patientRole.id.extension)
+2. Value of the header variable 'X-TechBD-CIN'
+3. Content of first occurance of the Location section from 
+Document.componentOf.encompassingEncounter.location.healthCareFacility.location OR 
+Document.component.structuredBody.component.section[code.code='46240-8'].entry[0].encounter.participant.participantRole</t>
+  </si>
+  <si>
+    <t>"id" : "ee527672b24d75f35b1773369ce2e357d31697b5deca4fee12d9518476f2ed",</t>
   </si>
   <si>
     <t>"http://hl7.org/fhir/us/sdoh-clinicalcare/StructureDefinition/SDOHCC-Location"</t>
@@ -5819,7 +5748,7 @@
     <numFmt numFmtId="178" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
     <numFmt numFmtId="179" formatCode="_ &quot;₹&quot;* #,##0_ ;_ &quot;₹&quot;* \-#,##0_ ;_ &quot;₹&quot;* &quot;-&quot;_ ;_ @_ "/>
   </numFmts>
-  <fonts count="41">
+  <fonts count="37">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -6069,8 +5998,9 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <b/>
+      <i/>
       <sz val="11"/>
+      <color rgb="FF00B050"/>
       <name val="Calibri"/>
       <charset val="134"/>
       <scheme val="minor"/>
@@ -6086,44 +6016,17 @@
     <font>
       <b/>
       <sz val="11"/>
-      <color rgb="FFFF0000"/>
-      <name val="Calibri"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <i/>
-      <sz val="11"/>
-      <color rgb="FF00B050"/>
       <name val="Calibri"/>
       <charset val="134"/>
       <scheme val="minor"/>
     </font>
     <font>
       <b/>
-      <sz val="9"/>
-      <color rgb="FF00B050"/>
-      <name val="Consolas"/>
+      <sz val="11"/>
+      <color rgb="FFFF0000"/>
+      <name val="Calibri"/>
       <charset val="134"/>
-    </font>
-    <font>
-      <sz val="9"/>
-      <color rgb="FF00B050"/>
-      <name val="Consolas"/>
-      <charset val="134"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="10.5"/>
-      <color rgb="FF00B050"/>
-      <name val="Segoe UI"/>
-      <charset val="134"/>
-    </font>
-    <font>
-      <sz val="10.5"/>
-      <color rgb="FF00B050"/>
-      <name val="Segoe UI"/>
-      <charset val="134"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="35">
@@ -6588,7 +6491,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="35">
+  <cellXfs count="36">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -6606,6 +6509,9 @@
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1">
       <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
@@ -6673,6 +6579,9 @@
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
@@ -6689,9 +6598,6 @@
       <alignment horizontal="center" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1" quotePrefix="1">
@@ -7231,20 +7137,20 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
   <dimension ref="A1:C7"/>
-  <sheetFormatPr defaultColWidth="8.88181818181818" defaultRowHeight="14.5" outlineLevelRow="6" outlineLevelCol="2"/>
+  <sheetFormatPr defaultColWidth="8.88571428571429" defaultRowHeight="15" outlineLevelRow="6" outlineLevelCol="2"/>
   <cols>
-    <col min="1" max="1" width="8.88181818181818" style="32"/>
-    <col min="2" max="2" width="35.2181818181818" customWidth="1"/>
-    <col min="3" max="3" width="92.6636363636364" customWidth="1"/>
+    <col min="1" max="1" width="8.88571428571429" style="34"/>
+    <col min="2" max="2" width="35.2190476190476" customWidth="1"/>
+    <col min="3" max="3" width="92.6666666666667" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3">
-      <c r="B1" s="33" t="s">
+      <c r="B1" s="35" t="s">
         <v>0</v>
       </c>
     </row>
     <row r="3" spans="1:3">
-      <c r="A3" s="32">
+      <c r="A3" s="34">
         <v>1</v>
       </c>
       <c r="B3" s="5" t="s">
@@ -7255,10 +7161,10 @@
       </c>
     </row>
     <row r="4" spans="1:3">
-      <c r="A4" s="32">
+      <c r="A4" s="34">
         <v>2</v>
       </c>
-      <c r="B4" s="9" t="s">
+      <c r="B4" s="10" t="s">
         <v>3</v>
       </c>
       <c r="C4" t="s">
@@ -7266,10 +7172,10 @@
       </c>
     </row>
     <row r="5" spans="1:3">
-      <c r="A5" s="32">
+      <c r="A5" s="34">
         <v>3</v>
       </c>
-      <c r="B5" s="19" t="s">
+      <c r="B5" s="20" t="s">
         <v>3</v>
       </c>
       <c r="C5" t="s">
@@ -7277,10 +7183,10 @@
       </c>
     </row>
     <row r="6" spans="1:3">
-      <c r="A6" s="32">
+      <c r="A6" s="34">
         <v>4</v>
       </c>
-      <c r="B6" s="26" t="s">
+      <c r="B6" s="27" t="s">
         <v>3</v>
       </c>
       <c r="C6" t="s">
@@ -7288,10 +7194,10 @@
       </c>
     </row>
     <row r="7" spans="1:3">
-      <c r="A7" s="32">
+      <c r="A7" s="34">
         <v>5</v>
       </c>
-      <c r="B7" s="34" t="s">
+      <c r="B7" s="29" t="s">
         <v>3</v>
       </c>
       <c r="C7" t="s">
@@ -7308,14 +7214,14 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
   <dimension ref="A1:G17"/>
-  <sheetFormatPr defaultColWidth="9.14545454545454" defaultRowHeight="14.5" outlineLevelCol="6"/>
+  <sheetFormatPr defaultColWidth="9.14285714285714" defaultRowHeight="15" outlineLevelCol="6"/>
   <cols>
-    <col min="1" max="1" width="14.7181818181818" customWidth="1"/>
-    <col min="2" max="2" width="30.8545454545455" customWidth="1"/>
-    <col min="3" max="3" width="63.4272727272727" customWidth="1"/>
-    <col min="4" max="4" width="70.7181818181818" customWidth="1"/>
-    <col min="5" max="5" width="52.4272727272727" customWidth="1"/>
-    <col min="6" max="6" width="57.5727272727273" customWidth="1"/>
+    <col min="1" max="1" width="14.7142857142857" customWidth="1"/>
+    <col min="2" max="2" width="30.8571428571429" customWidth="1"/>
+    <col min="3" max="3" width="63.4285714285714" customWidth="1"/>
+    <col min="4" max="4" width="70.7142857142857" customWidth="1"/>
+    <col min="5" max="5" width="52.4285714285714" customWidth="1"/>
+    <col min="6" max="6" width="57.5714285714286" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" s="1" customFormat="1" spans="1:7">
@@ -7343,7 +7249,7 @@
         <v>47</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>430</v>
+        <v>435</v>
       </c>
       <c r="C2" s="3"/>
       <c r="D2" s="3"/>
@@ -7354,164 +7260,165 @@
         <v>14</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>431</v>
-      </c>
-    </row>
-    <row r="4" ht="58" spans="1:7">
+        <v>436</v>
+      </c>
+    </row>
+    <row r="4" ht="135" spans="1:7">
       <c r="B4" s="5" t="s">
         <v>16</v>
       </c>
-      <c r="C4" t="s">
-        <v>17</v>
-      </c>
-      <c r="E4" s="6" t="s">
-        <v>432</v>
-      </c>
-      <c r="F4" s="7"/>
-      <c r="G4" s="7"/>
+      <c r="C4" s="6" t="s">
+        <v>437</v>
+      </c>
+      <c r="D4" t="s">
+        <v>438</v>
+      </c>
+      <c r="E4" s="7"/>
+      <c r="F4" s="8"/>
+      <c r="G4" s="8"/>
     </row>
     <row r="5" spans="1:7">
       <c r="B5" s="5" t="s">
         <v>19</v>
       </c>
       <c r="C5" t="s">
-        <v>200</v>
-      </c>
-      <c r="E5" s="8"/>
-    </row>
-    <row r="6" ht="29" spans="1:7">
+        <v>201</v>
+      </c>
+      <c r="E5" s="9"/>
+    </row>
+    <row r="6" ht="30" spans="1:7">
       <c r="B6" s="5" t="s">
         <v>22</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>433</v>
+        <v>439</v>
       </c>
       <c r="E6" s="4" t="s">
-        <v>434</v>
-      </c>
-      <c r="F6" s="9" t="s">
-        <v>435</v>
+        <v>440</v>
+      </c>
+      <c r="F6" s="10" t="s">
+        <v>441</v>
       </c>
     </row>
     <row r="7" spans="1:7">
       <c r="B7" s="5" t="s">
-        <v>324</v>
-      </c>
-      <c r="C7" s="10" t="s">
-        <v>436</v>
+        <v>327</v>
+      </c>
+      <c r="C7" s="11" t="s">
+        <v>442</v>
       </c>
       <c r="D7" t="s">
-        <v>437</v>
-      </c>
-      <c r="E7" s="11"/>
+        <v>443</v>
+      </c>
+      <c r="E7" s="12"/>
       <c r="F7" s="4"/>
     </row>
-    <row r="8" customFormat="1" ht="72.5" spans="1:7">
+    <row r="8" customFormat="1" ht="75" spans="1:7">
       <c r="B8" s="4" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="C8" s="4" t="s">
-        <v>438</v>
-      </c>
-      <c r="D8" s="12" t="s">
-        <v>86</v>
-      </c>
-      <c r="E8" s="13" t="s">
-        <v>439</v>
-      </c>
-    </row>
-    <row r="9" customFormat="1" ht="58" spans="1:7">
+        <v>444</v>
+      </c>
+      <c r="D8" s="13" t="s">
+        <v>87</v>
+      </c>
+      <c r="E8" s="14" t="s">
+        <v>445</v>
+      </c>
+    </row>
+    <row r="9" customFormat="1" ht="60" spans="1:7">
       <c r="B9" s="4" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="C9" s="4" t="s">
-        <v>440</v>
-      </c>
-      <c r="D9" s="12"/>
+        <v>446</v>
+      </c>
+      <c r="D9" s="13"/>
       <c r="E9" s="4"/>
     </row>
     <row r="10" customFormat="1" spans="1:7">
       <c r="B10" s="4" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="C10" s="4" t="s">
-        <v>441</v>
-      </c>
-      <c r="D10" s="12"/>
+        <v>447</v>
+      </c>
+      <c r="D10" s="13"/>
       <c r="E10" s="4"/>
     </row>
     <row r="11" customFormat="1" spans="1:7">
       <c r="B11" s="4" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="C11" s="4" t="s">
-        <v>442</v>
-      </c>
-      <c r="D11" s="12"/>
+        <v>448</v>
+      </c>
+      <c r="D11" s="13"/>
       <c r="E11" s="4"/>
     </row>
     <row r="12" customFormat="1" spans="1:7">
       <c r="B12" s="4" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="C12" s="4" t="s">
-        <v>443</v>
-      </c>
-      <c r="D12" s="12"/>
+        <v>449</v>
+      </c>
+      <c r="D12" s="13"/>
       <c r="E12" s="4"/>
     </row>
     <row r="13" customFormat="1" spans="1:7">
       <c r="B13" s="4" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="C13" s="4" t="s">
-        <v>444</v>
-      </c>
-      <c r="D13" s="12"/>
+        <v>450</v>
+      </c>
+      <c r="D13" s="13"/>
       <c r="E13" s="4"/>
     </row>
     <row r="14" customFormat="1" spans="1:7">
       <c r="B14" s="4" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="C14" s="4" t="s">
-        <v>445</v>
-      </c>
-      <c r="D14" s="12"/>
+        <v>451</v>
+      </c>
+      <c r="D14" s="13"/>
       <c r="E14" s="4"/>
     </row>
     <row r="15" customFormat="1" spans="1:7">
       <c r="B15" s="4" t="s">
-        <v>446</v>
+        <v>452</v>
       </c>
       <c r="C15" s="4" t="s">
-        <v>447</v>
-      </c>
-      <c r="D15" s="12"/>
+        <v>453</v>
+      </c>
+      <c r="D15" s="13"/>
       <c r="E15" s="4"/>
     </row>
     <row r="16" customFormat="1" spans="1:7">
       <c r="B16" s="4" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="C16" s="4" t="s">
-        <v>193</v>
-      </c>
-      <c r="D16" s="14" t="s">
-        <v>448</v>
-      </c>
-      <c r="E16" s="8"/>
+        <v>194</v>
+      </c>
+      <c r="D16" s="15" t="s">
+        <v>454</v>
+      </c>
+      <c r="E16" s="9"/>
       <c r="F16" s="4"/>
     </row>
     <row r="17" customFormat="1" ht="60" customHeight="1" spans="2:6">
       <c r="B17" s="4" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="C17" s="4" t="s">
-        <v>449</v>
-      </c>
-      <c r="D17" s="14"/>
-      <c r="E17" s="8"/>
+        <v>455</v>
+      </c>
+      <c r="D17" s="15"/>
+      <c r="E17" s="9"/>
       <c r="F17" s="4"/>
     </row>
   </sheetData>
@@ -7529,14 +7436,14 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
   <dimension ref="A1:F22"/>
-  <sheetFormatPr defaultColWidth="9.14545454545454" defaultRowHeight="14.5" outlineLevelCol="5"/>
+  <sheetFormatPr defaultColWidth="9.14285714285714" defaultRowHeight="15" outlineLevelCol="5"/>
   <cols>
-    <col min="1" max="1" width="14.7181818181818" customWidth="1"/>
-    <col min="2" max="2" width="28.3363636363636" customWidth="1"/>
-    <col min="3" max="3" width="65.6636363636364" customWidth="1"/>
-    <col min="4" max="4" width="46.2181818181818" customWidth="1"/>
-    <col min="5" max="5" width="61.2818181818182" customWidth="1"/>
-    <col min="6" max="6" width="46.2818181818182" customWidth="1"/>
+    <col min="1" max="1" width="14.7142857142857" customWidth="1"/>
+    <col min="2" max="2" width="28.3333333333333" customWidth="1"/>
+    <col min="3" max="3" width="65.6666666666667" customWidth="1"/>
+    <col min="4" max="4" width="46.2190476190476" customWidth="1"/>
+    <col min="5" max="5" width="61.2857142857143" customWidth="1"/>
+    <col min="6" max="6" width="46.2857142857143" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" s="1" customFormat="1" spans="1:6">
@@ -7578,44 +7485,44 @@
       <c r="B4" t="s">
         <v>16</v>
       </c>
-      <c r="C4" t="s">
+      <c r="C4" s="29" t="s">
         <v>17</v>
       </c>
       <c r="D4" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="5" s="27" customFormat="1" ht="61" customHeight="1" spans="1:6">
-      <c r="A5" s="28"/>
-      <c r="B5" s="28" t="s">
+    <row r="5" s="28" customFormat="1" ht="61" customHeight="1" spans="1:6">
+      <c r="A5" s="30"/>
+      <c r="B5" s="30" t="s">
         <v>19</v>
       </c>
-      <c r="C5" s="28" t="s">
+      <c r="C5" s="30" t="s">
         <v>20</v>
       </c>
-      <c r="D5" s="29" t="s">
+      <c r="D5" s="31" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="6" s="27" customFormat="1" ht="49" customHeight="1" spans="1:6">
-      <c r="A6" s="28"/>
-      <c r="B6" s="28" t="s">
+    <row r="6" s="28" customFormat="1" ht="49" customHeight="1" spans="1:6">
+      <c r="A6" s="30"/>
+      <c r="B6" s="30" t="s">
         <v>22</v>
       </c>
-      <c r="C6" s="28" t="s">
+      <c r="C6" s="30" t="s">
         <v>23</v>
       </c>
-      <c r="D6" s="29"/>
-    </row>
-    <row r="7" s="27" customFormat="1" ht="316" customHeight="1" spans="1:6">
-      <c r="A7" s="28"/>
-      <c r="B7" s="28" t="s">
+      <c r="D6" s="31"/>
+    </row>
+    <row r="7" s="28" customFormat="1" ht="316" customHeight="1" spans="1:6">
+      <c r="A7" s="30"/>
+      <c r="B7" s="30" t="s">
         <v>24</v>
       </c>
-      <c r="C7" s="30" t="s">
+      <c r="C7" s="32" t="s">
         <v>25</v>
       </c>
-      <c r="D7" s="29"/>
+      <c r="D7" s="31"/>
     </row>
     <row r="8" customFormat="1" spans="1:6">
       <c r="B8" t="s">
@@ -7634,7 +7541,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="10" customFormat="1" ht="29" spans="1:6">
+    <row r="10" customFormat="1" ht="30" spans="1:6">
       <c r="B10" t="s">
         <v>30</v>
       </c>
@@ -7655,11 +7562,11 @@
         <v>34</v>
       </c>
     </row>
-    <row r="16" ht="72.5" spans="1:6">
+    <row r="16" ht="75" spans="1:6">
       <c r="B16" t="s">
         <v>35</v>
       </c>
-      <c r="C16" s="10" t="s">
+      <c r="C16" s="11" t="s">
         <v>36</v>
       </c>
     </row>
@@ -7671,46 +7578,46 @@
         <v>38</v>
       </c>
     </row>
-    <row r="18" ht="72.5" spans="2:5">
+    <row r="18" ht="75" spans="2:5">
       <c r="B18" t="s">
         <v>39</v>
       </c>
       <c r="C18" t="s">
         <v>40</v>
       </c>
-      <c r="E18" s="18" t="s">
+      <c r="E18" s="19" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="19" ht="29" spans="2:5">
+    <row r="19" ht="45" spans="2:5">
       <c r="B19" s="4" t="s">
         <v>42</v>
       </c>
-      <c r="C19" s="10" t="s">
+      <c r="C19" s="11" t="s">
         <v>43</v>
       </c>
-      <c r="E19" s="10"/>
-    </row>
-    <row r="20" ht="43.5" spans="2:5">
+      <c r="E19" s="11"/>
+    </row>
+    <row r="20" ht="45" spans="2:5">
       <c r="B20" t="s">
         <v>44</v>
       </c>
-      <c r="C20" s="10" t="s">
+      <c r="C20" s="11" t="s">
         <v>45</v>
       </c>
-      <c r="E20" s="10"/>
-    </row>
-    <row r="21" ht="29" spans="2:5">
+      <c r="E20" s="11"/>
+    </row>
+    <row r="21" ht="30" spans="2:5">
       <c r="B21" s="4" t="s">
         <v>46</v>
       </c>
-      <c r="E21" s="8"/>
-    </row>
-    <row r="22" ht="101.5" spans="2:5">
-      <c r="B22" s="31" t="s">
+      <c r="E21" s="9"/>
+    </row>
+    <row r="22" ht="105" spans="2:5">
+      <c r="B22" s="33" t="s">
         <v>47</v>
       </c>
-      <c r="C22" s="10" t="s">
+      <c r="C22" s="11" t="s">
         <v>48</v>
       </c>
     </row>
@@ -7730,13 +7637,13 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
   <dimension ref="A1:F68"/>
-  <sheetFormatPr defaultColWidth="8.88181818181818" defaultRowHeight="14.5" outlineLevelCol="5"/>
+  <sheetFormatPr defaultColWidth="8.88571428571429" defaultRowHeight="15" outlineLevelCol="5"/>
   <cols>
-    <col min="1" max="1" width="14.7181818181818" customWidth="1"/>
-    <col min="2" max="2" width="41.7818181818182" style="4" customWidth="1"/>
-    <col min="3" max="3" width="63.8818181818182" style="4" customWidth="1"/>
-    <col min="4" max="4" width="81.2818181818182" style="4" customWidth="1"/>
-    <col min="5" max="5" width="48.4272727272727" style="4" customWidth="1"/>
+    <col min="1" max="1" width="14.7142857142857" customWidth="1"/>
+    <col min="2" max="2" width="41.7809523809524" style="4" customWidth="1"/>
+    <col min="3" max="3" width="63.8857142857143" style="4" customWidth="1"/>
+    <col min="4" max="4" width="81.2857142857143" style="4" customWidth="1"/>
+    <col min="5" max="5" width="48.4285714285714" style="4" customWidth="1"/>
     <col min="6" max="6" width="45" customWidth="1"/>
   </cols>
   <sheetData>
@@ -7744,19 +7651,19 @@
       <c r="A1" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="B1" s="24" t="s">
+      <c r="B1" s="25" t="s">
         <v>9</v>
       </c>
-      <c r="C1" s="24" t="s">
+      <c r="C1" s="25" t="s">
         <v>10</v>
       </c>
-      <c r="D1" s="24" t="s">
+      <c r="D1" s="25" t="s">
         <v>11</v>
       </c>
-      <c r="E1" s="24" t="s">
+      <c r="E1" s="25" t="s">
         <v>49</v>
       </c>
-      <c r="F1" s="24" t="s">
+      <c r="F1" s="25" t="s">
         <v>50</v>
       </c>
     </row>
@@ -7774,685 +7681,685 @@
         <v>51</v>
       </c>
     </row>
-    <row r="4" spans="1:6">
-      <c r="B4" s="15" t="s">
+    <row r="4" ht="90" spans="1:6">
+      <c r="B4" s="16" t="s">
         <v>16</v>
       </c>
-      <c r="C4" s="4" t="s">
-        <v>17</v>
+      <c r="C4" s="19" t="s">
+        <v>52</v>
       </c>
       <c r="D4" s="4" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
     </row>
     <row r="5" spans="1:6">
       <c r="A5" s="1"/>
-      <c r="B5" s="15" t="s">
+      <c r="B5" s="16" t="s">
         <v>19</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
     </row>
     <row r="6" spans="1:6">
-      <c r="B6" s="15" t="s">
+      <c r="B6" s="16" t="s">
         <v>22</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="7" ht="29" spans="1:6">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="7" ht="30" spans="1:6">
       <c r="B7" s="4" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="C7" s="4" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="D7" s="4" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="8" ht="58" spans="1:6">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="8" ht="60" spans="1:6">
       <c r="B8" s="4" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="C8" s="4" t="s">
-        <v>59</v>
-      </c>
-      <c r="D8" s="10" t="s">
         <v>60</v>
       </c>
+      <c r="D8" s="11" t="s">
+        <v>61</v>
+      </c>
       <c r="E8" s="4" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
     </row>
     <row r="9" spans="1:6">
-      <c r="B9" s="10" t="s">
-        <v>62</v>
+      <c r="B9" s="11" t="s">
+        <v>63</v>
       </c>
       <c r="C9" s="4" t="s">
-        <v>63</v>
-      </c>
-      <c r="D9" s="10"/>
+        <v>64</v>
+      </c>
+      <c r="D9" s="11"/>
     </row>
     <row r="10" spans="1:6">
       <c r="B10" s="4" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="C10" s="4" t="s">
-        <v>65</v>
-      </c>
-      <c r="D10" s="10" t="s">
         <v>66</v>
       </c>
+      <c r="D10" s="11" t="s">
+        <v>67</v>
+      </c>
     </row>
     <row r="11" spans="1:6">
-      <c r="B11" s="15" t="s">
-        <v>67</v>
+      <c r="B11" s="16" t="s">
+        <v>68</v>
       </c>
       <c r="C11" s="4" t="s">
-        <v>68</v>
-      </c>
-      <c r="D11" s="10" t="s">
         <v>69</v>
       </c>
+      <c r="D11" s="11" t="s">
+        <v>70</v>
+      </c>
     </row>
     <row r="12" spans="1:6">
-      <c r="B12" s="15" t="s">
-        <v>70</v>
+      <c r="B12" s="16" t="s">
+        <v>71</v>
       </c>
       <c r="C12" s="4" t="s">
-        <v>59</v>
-      </c>
-      <c r="D12" s="10" t="s">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="13" ht="58" spans="1:6">
+        <v>60</v>
+      </c>
+      <c r="D12" s="11" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="13" ht="60" spans="1:6">
       <c r="B13" s="4" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="C13" s="4" t="s">
-        <v>73</v>
-      </c>
-      <c r="D13" s="10" t="s">
         <v>74</v>
       </c>
-    </row>
-    <row r="14" ht="29" spans="1:6">
+      <c r="D13" s="11" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="14" ht="30" spans="1:6">
       <c r="B14" s="4" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="C14" s="4" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="D14" s="4" t="s">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="15" ht="29" spans="1:6">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="15" ht="30" spans="1:6">
       <c r="B15" s="4" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="C15" s="4" t="s">
-        <v>79</v>
-      </c>
-      <c r="D15" s="10" t="s">
         <v>80</v>
       </c>
+      <c r="D15" s="11" t="s">
+        <v>81</v>
+      </c>
     </row>
     <row r="16" spans="1:6">
-      <c r="B16" s="15" t="s">
-        <v>81</v>
+      <c r="B16" s="16" t="s">
+        <v>82</v>
       </c>
       <c r="C16" s="4" t="s">
-        <v>82</v>
-      </c>
-      <c r="D16" s="10" t="s">
         <v>83</v>
       </c>
-    </row>
-    <row r="17" ht="72.5" spans="2:5">
+      <c r="D16" s="11" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="17" ht="75" spans="2:5">
       <c r="B17" s="4" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="C17" s="4" t="s">
-        <v>85</v>
-      </c>
-      <c r="D17" s="12" t="s">
         <v>86</v>
       </c>
-      <c r="E17" s="13" t="s">
+      <c r="D17" s="13" t="s">
         <v>87</v>
       </c>
-    </row>
-    <row r="18" ht="58" spans="2:5">
+      <c r="E17" s="14" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="18" ht="60" spans="2:5">
       <c r="B18" s="4" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="C18" s="4" t="s">
-        <v>89</v>
-      </c>
-      <c r="D18" s="12"/>
+        <v>90</v>
+      </c>
+      <c r="D18" s="13"/>
     </row>
     <row r="19" spans="2:5">
       <c r="B19" s="4" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="C19" s="4" t="s">
-        <v>91</v>
-      </c>
-      <c r="D19" s="12"/>
+        <v>92</v>
+      </c>
+      <c r="D19" s="13"/>
     </row>
     <row r="20" spans="2:5">
       <c r="B20" s="4" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="C20" s="4" t="s">
-        <v>93</v>
-      </c>
-      <c r="D20" s="12"/>
+        <v>94</v>
+      </c>
+      <c r="D20" s="13"/>
     </row>
     <row r="21" spans="2:5">
       <c r="B21" s="4" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="C21" s="4" t="s">
-        <v>95</v>
-      </c>
-      <c r="D21" s="12"/>
+        <v>96</v>
+      </c>
+      <c r="D21" s="13"/>
     </row>
     <row r="22" spans="2:5">
       <c r="B22" s="4" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="C22" s="4" t="s">
-        <v>97</v>
-      </c>
-      <c r="D22" s="12"/>
+        <v>98</v>
+      </c>
+      <c r="D22" s="13"/>
     </row>
     <row r="23" spans="2:5">
       <c r="B23" s="4" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="C23" s="4" t="s">
-        <v>99</v>
-      </c>
-      <c r="D23" s="12"/>
-    </row>
-    <row r="24" ht="116" spans="2:5">
+        <v>100</v>
+      </c>
+      <c r="D23" s="13"/>
+    </row>
+    <row r="24" ht="120" spans="2:5">
       <c r="B24" s="4" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="D24" s="4" t="s">
-        <v>101</v>
-      </c>
-      <c r="E24" s="18" t="s">
         <v>102</v>
+      </c>
+      <c r="E24" s="19" t="s">
+        <v>103</v>
       </c>
     </row>
     <row r="25" spans="2:5">
       <c r="B25" s="4" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="C25" s="4" t="s">
-        <v>104</v>
-      </c>
-    </row>
-    <row r="26" ht="87" spans="2:5">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="26" ht="90" spans="2:5">
       <c r="B26" s="4" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="C26" s="4" t="s">
-        <v>106</v>
-      </c>
-      <c r="E26" s="23" t="s">
         <v>107</v>
       </c>
-    </row>
-    <row r="27" ht="43.5" spans="2:5">
+      <c r="E26" s="24" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="27" ht="45" spans="2:5">
       <c r="B27" s="4" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="C27" s="4" t="s">
-        <v>109</v>
-      </c>
-      <c r="D27" s="12" t="s">
         <v>110</v>
       </c>
-      <c r="E27" s="8" t="s">
+      <c r="D27" s="13" t="s">
         <v>111</v>
       </c>
-    </row>
-    <row r="28" spans="2:5">
+      <c r="E27" s="9" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="28" ht="30" spans="2:5">
       <c r="B28" s="4" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="C28" s="4" t="s">
-        <v>113</v>
-      </c>
-      <c r="D28" s="14"/>
-      <c r="E28" s="8"/>
+        <v>114</v>
+      </c>
+      <c r="D28" s="15"/>
+      <c r="E28" s="9"/>
     </row>
     <row r="29" spans="2:5">
       <c r="B29" s="4" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="C29" s="4" t="s">
-        <v>115</v>
-      </c>
-      <c r="D29" s="14"/>
-      <c r="E29" s="8"/>
-    </row>
-    <row r="30" spans="2:5">
+        <v>116</v>
+      </c>
+      <c r="D29" s="15"/>
+      <c r="E29" s="9"/>
+    </row>
+    <row r="30" ht="30" spans="2:5">
       <c r="B30" s="4" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="C30" s="4" t="s">
-        <v>117</v>
-      </c>
-      <c r="D30" s="14"/>
-      <c r="E30" s="8"/>
+        <v>118</v>
+      </c>
+      <c r="D30" s="15"/>
+      <c r="E30" s="9"/>
     </row>
     <row r="31" spans="2:5">
       <c r="B31" s="4" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="C31" s="4" t="s">
-        <v>119</v>
-      </c>
-      <c r="D31" s="14"/>
-      <c r="E31" s="8"/>
-    </row>
-    <row r="32" ht="43.5" spans="2:5">
+        <v>120</v>
+      </c>
+      <c r="D31" s="15"/>
+      <c r="E31" s="9"/>
+    </row>
+    <row r="32" ht="45" spans="2:5">
       <c r="B32" s="4" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="C32" s="4" t="s">
-        <v>109</v>
-      </c>
-      <c r="D32" s="14" t="s">
-        <v>120</v>
-      </c>
-      <c r="E32" s="8" t="s">
+        <v>110</v>
+      </c>
+      <c r="D32" s="15" t="s">
         <v>121</v>
       </c>
-    </row>
-    <row r="33" spans="2:6">
+      <c r="E32" s="9" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="33" ht="30" spans="2:6">
       <c r="B33" s="4" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="C33" s="4" t="s">
-        <v>122</v>
-      </c>
-      <c r="D33" s="14"/>
+        <v>123</v>
+      </c>
+      <c r="D33" s="15"/>
     </row>
     <row r="34" spans="2:6">
       <c r="B34" s="4" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="C34" s="4" t="s">
-        <v>123</v>
-      </c>
-      <c r="D34" s="14"/>
-    </row>
-    <row r="35" spans="2:6">
+        <v>124</v>
+      </c>
+      <c r="D34" s="15"/>
+    </row>
+    <row r="35" ht="30" spans="2:6">
       <c r="B35" s="4" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="C35" s="4" t="s">
-        <v>124</v>
-      </c>
-      <c r="D35" s="14"/>
+        <v>125</v>
+      </c>
+      <c r="D35" s="15"/>
     </row>
     <row r="36" spans="2:6">
       <c r="B36" s="4" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="C36" s="4" t="s">
-        <v>125</v>
-      </c>
-      <c r="D36" s="14"/>
+        <v>126</v>
+      </c>
+      <c r="D36" s="15"/>
     </row>
     <row r="37" spans="2:6">
       <c r="B37" s="4" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="C37" s="4" t="s">
-        <v>126</v>
-      </c>
-      <c r="D37" s="14" t="s">
         <v>127</v>
       </c>
-    </row>
-    <row r="38" ht="43.5" spans="2:6">
+      <c r="D37" s="15" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="38" ht="45" spans="2:6">
       <c r="B38" s="4" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="C38" s="4" t="s">
-        <v>79</v>
-      </c>
-      <c r="D38" s="14"/>
-      <c r="E38" s="35" t="s">
-        <v>129</v>
-      </c>
-    </row>
-    <row r="39" ht="116" spans="2:6">
+        <v>80</v>
+      </c>
+      <c r="D38" s="15"/>
+      <c r="E38" s="36" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="39" ht="120" spans="2:6">
       <c r="B39" s="4" t="s">
-        <v>130</v>
-      </c>
-      <c r="D39" s="10" t="s">
         <v>131</v>
       </c>
+      <c r="D39" s="11" t="s">
+        <v>132</v>
+      </c>
       <c r="F39" s="4" t="s">
-        <v>132</v>
-      </c>
-    </row>
-    <row r="40" ht="116" spans="2:6">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="40" ht="120" spans="2:6">
       <c r="B40" s="4" t="s">
-        <v>133</v>
-      </c>
-      <c r="D40" s="10" t="s">
         <v>134</v>
       </c>
+      <c r="D40" s="11" t="s">
+        <v>135</v>
+      </c>
       <c r="F40" s="4" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
     </row>
     <row r="41" spans="2:6">
-      <c r="B41" s="15" t="s">
-        <v>136</v>
+      <c r="B41" s="16" t="s">
+        <v>137</v>
       </c>
       <c r="C41" s="4" t="s">
-        <v>137</v>
-      </c>
-      <c r="D41" s="10"/>
+        <v>138</v>
+      </c>
+      <c r="D41" s="11"/>
     </row>
     <row r="42" spans="2:6">
-      <c r="B42" s="15" t="s">
-        <v>138</v>
+      <c r="B42" s="16" t="s">
+        <v>139</v>
       </c>
       <c r="C42" s="4" t="s">
-        <v>139</v>
-      </c>
-      <c r="D42" s="10"/>
+        <v>140</v>
+      </c>
+      <c r="D42" s="11"/>
     </row>
     <row r="43" spans="2:6">
-      <c r="B43" s="15" t="s">
-        <v>140</v>
+      <c r="B43" s="16" t="s">
+        <v>141</v>
       </c>
       <c r="C43" s="4" t="s">
-        <v>141</v>
-      </c>
-      <c r="D43" s="10"/>
+        <v>142</v>
+      </c>
+      <c r="D43" s="11"/>
     </row>
     <row r="44" spans="2:6">
       <c r="B44" s="4" t="s">
+        <v>143</v>
+      </c>
+      <c r="C44" s="4" t="s">
         <v>142</v>
       </c>
-      <c r="C44" s="4" t="s">
-        <v>141</v>
-      </c>
-      <c r="D44" s="10"/>
-    </row>
-    <row r="45" ht="188.5" spans="2:6">
-      <c r="B45" s="15" t="s">
-        <v>143</v>
-      </c>
-      <c r="C45" s="10" t="s">
+      <c r="D44" s="11"/>
+    </row>
+    <row r="45" ht="195" spans="2:6">
+      <c r="B45" s="16" t="s">
         <v>144</v>
       </c>
-      <c r="D45" s="10" t="s">
+      <c r="C45" s="11" t="s">
         <v>145</v>
       </c>
-      <c r="E45" s="18" t="s">
+      <c r="D45" s="11" t="s">
         <v>146</v>
       </c>
-    </row>
-    <row r="46" ht="188.5" spans="2:6">
-      <c r="B46" s="15" t="s">
+      <c r="E45" s="19" t="s">
         <v>147</v>
       </c>
-      <c r="C46" s="18" t="s">
+    </row>
+    <row r="46" ht="195" spans="2:6">
+      <c r="B46" s="16" t="s">
         <v>148</v>
       </c>
-      <c r="D46" s="10" t="s">
+      <c r="C46" s="19" t="s">
         <v>149</v>
       </c>
-      <c r="E46" s="8" t="s">
+      <c r="D46" s="11" t="s">
         <v>150</v>
       </c>
-    </row>
-    <row r="47" ht="188.5" spans="2:6">
-      <c r="B47" s="15" t="s">
+      <c r="E46" s="9" t="s">
         <v>151</v>
       </c>
+    </row>
+    <row r="47" ht="195" spans="2:6">
+      <c r="B47" s="16" t="s">
+        <v>152</v>
+      </c>
       <c r="C47" s="4" t="s">
-        <v>152</v>
-      </c>
-      <c r="D47" s="10" t="s">
         <v>153</v>
       </c>
-      <c r="E47" s="25"/>
+      <c r="D47" s="11" t="s">
+        <v>154</v>
+      </c>
+      <c r="E47" s="26"/>
     </row>
     <row r="48" customFormat="1" spans="2:6">
       <c r="B48" s="4" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="C48" s="4" t="s">
-        <v>137</v>
-      </c>
-      <c r="D48" s="10"/>
+        <v>138</v>
+      </c>
+      <c r="D48" s="11"/>
       <c r="E48" s="4"/>
     </row>
     <row r="49" customFormat="1" spans="2:6">
       <c r="B49" s="4" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="C49" s="4" t="s">
-        <v>156</v>
-      </c>
-      <c r="D49" s="10"/>
+        <v>157</v>
+      </c>
+      <c r="D49" s="11"/>
       <c r="E49" s="4"/>
     </row>
     <row r="50" customFormat="1" spans="2:6">
       <c r="B50" s="4" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="C50" s="4" t="s">
-        <v>158</v>
-      </c>
-      <c r="D50" s="10"/>
+        <v>159</v>
+      </c>
+      <c r="D50" s="11"/>
       <c r="E50" s="4"/>
     </row>
     <row r="51" customFormat="1" spans="2:6">
       <c r="B51" s="4" t="s">
+        <v>160</v>
+      </c>
+      <c r="C51" s="4" t="s">
         <v>159</v>
       </c>
-      <c r="C51" s="4" t="s">
-        <v>158</v>
-      </c>
-      <c r="D51" s="10"/>
+      <c r="D51" s="11"/>
       <c r="E51" s="4"/>
     </row>
-    <row r="52" ht="145" spans="2:6">
-      <c r="B52" s="10" t="s">
-        <v>160</v>
-      </c>
-      <c r="C52" s="18" t="s">
+    <row r="52" ht="150" spans="2:6">
+      <c r="B52" s="11" t="s">
         <v>161</v>
       </c>
-      <c r="D52" s="10" t="s">
+      <c r="C52" s="19" t="s">
         <v>162</v>
       </c>
-      <c r="E52" s="8" t="s">
+      <c r="D52" s="11" t="s">
         <v>163</v>
+      </c>
+      <c r="E52" s="9" t="s">
+        <v>164</v>
       </c>
     </row>
     <row r="53" spans="2:6">
       <c r="B53" s="4" t="s">
-        <v>164</v>
-      </c>
-      <c r="C53" s="10" t="s">
         <v>165</v>
       </c>
-      <c r="D53" s="10"/>
-      <c r="E53" s="8"/>
+      <c r="C53" s="11" t="s">
+        <v>166</v>
+      </c>
+      <c r="D53" s="11"/>
+      <c r="E53" s="9"/>
     </row>
     <row r="54" customFormat="1" spans="2:6">
       <c r="B54" s="4" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="C54" s="4" t="s">
-        <v>137</v>
-      </c>
-      <c r="D54" s="10"/>
-      <c r="E54" s="8"/>
+        <v>138</v>
+      </c>
+      <c r="D54" s="11"/>
+      <c r="E54" s="9"/>
     </row>
     <row r="55" customFormat="1" spans="2:6">
       <c r="B55" s="4" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="C55" s="4" t="s">
-        <v>168</v>
-      </c>
-      <c r="D55" s="10"/>
-      <c r="E55" s="8"/>
+        <v>169</v>
+      </c>
+      <c r="D55" s="11"/>
+      <c r="E55" s="9"/>
     </row>
     <row r="56" customFormat="1" spans="2:6">
       <c r="B56" s="4" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="C56" s="4" t="s">
-        <v>170</v>
-      </c>
-      <c r="D56" s="10"/>
-      <c r="E56" s="8"/>
+        <v>171</v>
+      </c>
+      <c r="D56" s="11"/>
+      <c r="E56" s="9"/>
     </row>
     <row r="57" customFormat="1" spans="2:6">
       <c r="B57" s="4" t="s">
+        <v>172</v>
+      </c>
+      <c r="C57" s="4" t="s">
         <v>171</v>
       </c>
-      <c r="C57" s="4" t="s">
-        <v>170</v>
-      </c>
-      <c r="D57" s="10"/>
-      <c r="E57" s="8"/>
+      <c r="D57" s="11"/>
+      <c r="E57" s="9"/>
     </row>
     <row r="58" spans="2:6">
       <c r="B58" s="4" t="s">
-        <v>172</v>
-      </c>
-      <c r="C58" s="10" t="s">
         <v>173</v>
       </c>
-      <c r="D58" s="10"/>
-      <c r="E58" s="8"/>
-    </row>
-    <row r="59" ht="174" spans="2:6">
-      <c r="B59" s="10" t="s">
+      <c r="C58" s="11" t="s">
         <v>174</v>
       </c>
-      <c r="C59" s="10" t="s">
-        <v>144</v>
-      </c>
-      <c r="D59" s="10" t="s">
+      <c r="D58" s="11"/>
+      <c r="E58" s="9"/>
+    </row>
+    <row r="59" ht="180" spans="2:6">
+      <c r="B59" s="11" t="s">
         <v>175</v>
       </c>
-      <c r="E59" s="18" t="s">
+      <c r="C59" s="11" t="s">
+        <v>145</v>
+      </c>
+      <c r="D59" s="11" t="s">
         <v>176</v>
       </c>
-    </row>
-    <row r="60" ht="246.5" spans="2:6">
+      <c r="E59" s="19" t="s">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="60" ht="255" spans="2:6">
       <c r="B60" s="4" t="s">
-        <v>177</v>
-      </c>
-      <c r="D60" s="10" t="s">
         <v>178</v>
       </c>
+      <c r="D60" s="11" t="s">
+        <v>179</v>
+      </c>
       <c r="F60" s="4" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
     </row>
     <row r="61" spans="2:6">
       <c r="B61" s="4" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="C61" s="4" t="s">
-        <v>181</v>
-      </c>
-      <c r="D61" s="10"/>
+        <v>182</v>
+      </c>
+      <c r="D61" s="11"/>
       <c r="F61" s="4"/>
     </row>
     <row r="62" spans="2:6">
       <c r="B62" s="4" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="C62" s="4" t="s">
-        <v>183</v>
-      </c>
-      <c r="D62" s="10"/>
+        <v>184</v>
+      </c>
+      <c r="D62" s="11"/>
       <c r="F62" s="4"/>
     </row>
-    <row r="63" ht="203" spans="2:6">
+    <row r="63" ht="210" spans="2:6">
       <c r="B63" s="4" t="s">
-        <v>184</v>
-      </c>
-      <c r="D63" s="10"/>
-      <c r="E63" s="13" t="s">
         <v>185</v>
+      </c>
+      <c r="D63" s="11"/>
+      <c r="E63" s="14" t="s">
+        <v>186</v>
       </c>
       <c r="F63" s="4"/>
     </row>
     <row r="64" ht="56" customHeight="1" spans="2:6">
       <c r="B64" s="4" t="s">
-        <v>186</v>
-      </c>
-      <c r="D64" s="12" t="s">
         <v>187</v>
       </c>
+      <c r="D64" s="13" t="s">
+        <v>188</v>
+      </c>
       <c r="F64" s="4" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
     </row>
     <row r="65" ht="43" customHeight="1" spans="2:4">
       <c r="B65" s="4" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="C65" s="4" t="s">
-        <v>56</v>
-      </c>
-      <c r="D65" s="12"/>
+        <v>57</v>
+      </c>
+      <c r="D65" s="13"/>
     </row>
     <row r="66" ht="40" customHeight="1" spans="2:4">
       <c r="B66" s="4" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="C66" s="4" t="s">
-        <v>191</v>
-      </c>
-      <c r="D66" s="12"/>
+        <v>192</v>
+      </c>
+      <c r="D66" s="13"/>
     </row>
     <row r="67" spans="2:4">
       <c r="B67" s="4" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="C67" s="4" t="s">
-        <v>193</v>
-      </c>
-      <c r="D67" s="14" t="s">
         <v>194</v>
+      </c>
+      <c r="D67" s="15" t="s">
+        <v>195</v>
       </c>
     </row>
     <row r="68" ht="43" customHeight="1" spans="2:4">
       <c r="B68" s="4" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="C68" s="4" t="s">
-        <v>196</v>
-      </c>
-      <c r="D68" s="14"/>
+        <v>197</v>
+      </c>
+      <c r="D68" s="15"/>
     </row>
   </sheetData>
   <mergeCells count="7">
@@ -8473,14 +8380,14 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
   <dimension ref="A1:G22"/>
-  <sheetFormatPr defaultColWidth="9.14545454545454" defaultRowHeight="14.5" outlineLevelCol="6"/>
+  <sheetFormatPr defaultColWidth="9.14285714285714" defaultRowHeight="15" outlineLevelCol="6"/>
   <cols>
-    <col min="1" max="1" width="14.7181818181818" customWidth="1"/>
-    <col min="2" max="2" width="30.8545454545455" customWidth="1"/>
-    <col min="3" max="3" width="63.4272727272727" customWidth="1"/>
-    <col min="4" max="4" width="70.7181818181818" customWidth="1"/>
-    <col min="5" max="5" width="52.4272727272727" customWidth="1"/>
-    <col min="6" max="6" width="57.5727272727273" customWidth="1"/>
+    <col min="1" max="1" width="14.7142857142857" customWidth="1"/>
+    <col min="2" max="2" width="30.8571428571429" customWidth="1"/>
+    <col min="3" max="3" width="63.4285714285714" customWidth="1"/>
+    <col min="4" max="4" width="70.7142857142857" customWidth="1"/>
+    <col min="5" max="5" width="52.4285714285714" customWidth="1"/>
+    <col min="6" max="6" width="57.5714285714286" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" s="1" customFormat="1" spans="1:7">
@@ -8508,7 +8415,7 @@
         <v>39</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="C2" s="3"/>
       <c r="D2" s="3"/>
@@ -8519,243 +8426,244 @@
         <v>14</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>198</v>
-      </c>
-    </row>
-    <row r="4" ht="58" spans="1:7">
+        <v>199</v>
+      </c>
+    </row>
+    <row r="4" ht="105" spans="1:7">
       <c r="B4" s="5" t="s">
         <v>16</v>
       </c>
-      <c r="C4" t="s">
-        <v>17</v>
-      </c>
-      <c r="E4" s="6" t="s">
-        <v>199</v>
-      </c>
-      <c r="F4" s="7"/>
-      <c r="G4" s="7"/>
+      <c r="C4" s="6" t="s">
+        <v>200</v>
+      </c>
+      <c r="D4" t="s">
+        <v>53</v>
+      </c>
+      <c r="E4" s="7"/>
+      <c r="F4" s="8"/>
+      <c r="G4" s="8"/>
     </row>
     <row r="5" spans="1:7">
       <c r="B5" s="5" t="s">
         <v>19</v>
       </c>
       <c r="C5" t="s">
-        <v>200</v>
-      </c>
-      <c r="E5" s="8"/>
+        <v>201</v>
+      </c>
+      <c r="E5" s="9"/>
     </row>
     <row r="6" spans="1:7">
       <c r="B6" s="5" t="s">
         <v>22</v>
       </c>
       <c r="C6" t="s">
-        <v>201</v>
-      </c>
-      <c r="E6" s="26"/>
-    </row>
-    <row r="7" ht="116" spans="1:7">
+        <v>202</v>
+      </c>
+      <c r="E6" s="27"/>
+    </row>
+    <row r="7" ht="120" spans="1:7">
       <c r="B7" s="5" t="s">
-        <v>202</v>
-      </c>
-      <c r="C7" s="10" t="s">
         <v>203</v>
       </c>
+      <c r="C7" s="11" t="s">
+        <v>204</v>
+      </c>
       <c r="D7" t="s">
-        <v>204</v>
-      </c>
-      <c r="E7" s="11" t="s">
         <v>205</v>
+      </c>
+      <c r="E7" s="12" t="s">
+        <v>206</v>
       </c>
       <c r="F7" s="4"/>
     </row>
     <row r="8" ht="94" customHeight="1" spans="1:7">
       <c r="B8" s="5" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="C8" t="s">
-        <v>207</v>
-      </c>
-      <c r="D8" s="10" t="s">
         <v>208</v>
       </c>
-      <c r="E8" s="8" t="s">
+      <c r="D8" s="11" t="s">
         <v>209</v>
+      </c>
+      <c r="E8" s="9" t="s">
+        <v>210</v>
       </c>
     </row>
     <row r="9" customFormat="1" spans="1:7">
       <c r="B9" s="5" t="s">
+        <v>211</v>
+      </c>
+      <c r="C9" t="s">
+        <v>212</v>
+      </c>
+      <c r="D9" s="11"/>
+      <c r="E9" s="9" t="s">
         <v>210</v>
-      </c>
-      <c r="C9" t="s">
-        <v>211</v>
-      </c>
-      <c r="D9" s="10"/>
-      <c r="E9" s="8" t="s">
-        <v>209</v>
       </c>
     </row>
     <row r="10" spans="1:7">
       <c r="B10" s="5" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="C10" t="s">
-        <v>213</v>
-      </c>
-      <c r="D10" s="10"/>
-      <c r="E10" s="8" t="s">
-        <v>209</v>
-      </c>
-    </row>
-    <row r="11" ht="203" spans="1:7">
+        <v>214</v>
+      </c>
+      <c r="D10" s="11"/>
+      <c r="E10" s="9" t="s">
+        <v>210</v>
+      </c>
+    </row>
+    <row r="11" ht="225" spans="1:7">
       <c r="B11" s="5" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="C11" t="s">
-        <v>215</v>
-      </c>
-      <c r="D11" s="10" t="s">
         <v>216</v>
       </c>
-      <c r="E11" s="8" t="s">
-        <v>209</v>
+      <c r="D11" s="11" t="s">
+        <v>217</v>
+      </c>
+      <c r="E11" s="9" t="s">
+        <v>210</v>
       </c>
     </row>
     <row r="12" spans="1:7">
       <c r="B12" s="5" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="C12" t="s">
-        <v>218</v>
-      </c>
-      <c r="E12" s="8" t="s">
-        <v>209</v>
+        <v>219</v>
+      </c>
+      <c r="E12" s="9" t="s">
+        <v>210</v>
       </c>
     </row>
     <row r="13" spans="1:7">
       <c r="B13" s="5" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
       <c r="C13" t="s">
-        <v>220</v>
-      </c>
-      <c r="E13" s="8" t="s">
-        <v>209</v>
-      </c>
-    </row>
-    <row r="14" ht="43.5" spans="1:7">
+        <v>221</v>
+      </c>
+      <c r="E13" s="9" t="s">
+        <v>210</v>
+      </c>
+    </row>
+    <row r="14" ht="45" spans="1:7">
       <c r="B14" s="5" t="s">
-        <v>221</v>
+        <v>222</v>
       </c>
       <c r="C14" s="4" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
       <c r="D14" t="s">
-        <v>223</v>
-      </c>
-      <c r="E14" s="8" t="s">
         <v>224</v>
       </c>
-    </row>
-    <row r="15" ht="246.5" spans="1:7">
+      <c r="E14" s="9" t="s">
+        <v>225</v>
+      </c>
+    </row>
+    <row r="15" ht="255" spans="1:7">
       <c r="B15" s="5" t="s">
-        <v>225</v>
-      </c>
-      <c r="C15" s="18" t="s">
         <v>226</v>
       </c>
-      <c r="D15" s="10" t="s">
+      <c r="C15" s="19" t="s">
         <v>227</v>
       </c>
-      <c r="E15" s="18" t="s">
+      <c r="D15" s="11" t="s">
         <v>228</v>
       </c>
-    </row>
-    <row r="16" ht="43.5" spans="1:7">
+      <c r="E15" s="19" t="s">
+        <v>229</v>
+      </c>
+    </row>
+    <row r="16" ht="45" spans="1:7">
       <c r="B16" s="5" t="s">
-        <v>229</v>
+        <v>230</v>
       </c>
       <c r="C16" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="D16" s="4" t="s">
-        <v>231</v>
-      </c>
-      <c r="E16" s="8"/>
-    </row>
-    <row r="17" ht="43.5" spans="2:6">
+        <v>232</v>
+      </c>
+      <c r="E16" s="9"/>
+    </row>
+    <row r="17" ht="45" spans="2:6">
       <c r="B17" s="5" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="C17" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="D17" s="4" t="s">
-        <v>234</v>
-      </c>
-      <c r="E17" s="8"/>
-    </row>
-    <row r="18" ht="43.5" spans="2:6">
+        <v>235</v>
+      </c>
+      <c r="E17" s="9"/>
+    </row>
+    <row r="18" ht="45" spans="2:6">
       <c r="B18" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
       <c r="C18" t="s">
-        <v>236</v>
-      </c>
-      <c r="D18" s="10" t="s">
         <v>237</v>
       </c>
-      <c r="E18" s="8" t="s">
-        <v>209</v>
-      </c>
-    </row>
-    <row r="19" ht="58" spans="2:6">
+      <c r="D18" s="11" t="s">
+        <v>238</v>
+      </c>
+      <c r="E18" s="9" t="s">
+        <v>210</v>
+      </c>
+    </row>
+    <row r="19" ht="60" spans="2:6">
       <c r="B19" s="5" t="s">
-        <v>238</v>
+        <v>239</v>
       </c>
       <c r="C19" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
       <c r="D19" s="4" t="s">
-        <v>240</v>
-      </c>
-      <c r="E19" s="8" t="s">
-        <v>209</v>
+        <v>241</v>
+      </c>
+      <c r="E19" s="9" t="s">
+        <v>210</v>
       </c>
     </row>
     <row r="20" customFormat="1" spans="2:6">
       <c r="B20" s="5" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="C20" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="D20" s="4"/>
-      <c r="E20" s="8" t="s">
-        <v>209</v>
+      <c r="E20" s="9" t="s">
+        <v>210</v>
       </c>
     </row>
     <row r="21" customFormat="1" spans="2:6">
       <c r="B21" s="4" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="C21" s="4" t="s">
-        <v>193</v>
-      </c>
-      <c r="D21" s="14" t="s">
-        <v>243</v>
-      </c>
-      <c r="E21" s="8"/>
+        <v>194</v>
+      </c>
+      <c r="D21" s="15" t="s">
+        <v>244</v>
+      </c>
+      <c r="E21" s="9"/>
       <c r="F21" s="4"/>
     </row>
     <row r="22" customFormat="1" ht="60" customHeight="1" spans="2:6">
       <c r="B22" s="4" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="C22" s="4" t="s">
-        <v>244</v>
-      </c>
-      <c r="D22" s="14"/>
-      <c r="E22" s="8"/>
+        <v>245</v>
+      </c>
+      <c r="D22" s="15"/>
+      <c r="E22" s="9"/>
       <c r="F22" s="4"/>
     </row>
   </sheetData>
@@ -8773,14 +8681,14 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
   <dimension ref="A1:F26"/>
-  <sheetFormatPr defaultColWidth="9.14545454545454" defaultRowHeight="14.5" outlineLevelCol="5"/>
+  <sheetFormatPr defaultColWidth="9.14285714285714" defaultRowHeight="15" outlineLevelCol="5"/>
   <cols>
-    <col min="1" max="1" width="14.7181818181818" customWidth="1"/>
-    <col min="2" max="2" width="35.1454545454545" customWidth="1"/>
-    <col min="3" max="3" width="42.2818181818182" style="4" customWidth="1"/>
-    <col min="4" max="4" width="73.5727272727273" customWidth="1"/>
+    <col min="1" max="1" width="14.7142857142857" customWidth="1"/>
+    <col min="2" max="2" width="35.1428571428571" customWidth="1"/>
+    <col min="3" max="3" width="52.7142857142857" style="4" customWidth="1"/>
+    <col min="4" max="4" width="73.5714285714286" customWidth="1"/>
     <col min="5" max="5" width="53" customWidth="1"/>
-    <col min="6" max="6" width="51.7181818181818" customWidth="1"/>
+    <col min="6" max="6" width="51.7142857142857" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" s="1" customFormat="1" spans="1:6">
@@ -8790,7 +8698,7 @@
       <c r="B1" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="C1" s="24" t="s">
+      <c r="C1" s="25" t="s">
         <v>10</v>
       </c>
       <c r="D1" s="2" t="s">
@@ -8808,7 +8716,7 @@
         <v>35</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="C2" s="3"/>
       <c r="D2" s="3"/>
@@ -8819,252 +8727,250 @@
         <v>14</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>246</v>
-      </c>
-    </row>
-    <row r="4" ht="72.5" spans="1:6">
+        <v>247</v>
+      </c>
+    </row>
+    <row r="4" ht="165" spans="1:6">
       <c r="A4" s="1"/>
       <c r="B4" s="5" t="s">
         <v>16</v>
       </c>
-      <c r="C4" s="4" t="s">
-        <v>17</v>
+      <c r="C4" s="19" t="s">
+        <v>248</v>
       </c>
       <c r="D4" t="s">
-        <v>247</v>
-      </c>
-      <c r="E4" s="8" t="s">
-        <v>248</v>
-      </c>
+        <v>249</v>
+      </c>
+      <c r="E4" s="9"/>
     </row>
     <row r="5" customFormat="1" spans="1:6">
       <c r="A5" s="1"/>
-      <c r="B5" s="15" t="s">
+      <c r="B5" s="16" t="s">
         <v>19</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="D5" s="4"/>
       <c r="E5" s="4"/>
       <c r="F5" s="4"/>
     </row>
-    <row r="6" customFormat="1" ht="29" spans="1:6">
-      <c r="B6" s="15" t="s">
+    <row r="6" customFormat="1" ht="30" spans="1:6">
+      <c r="B6" s="16" t="s">
         <v>22</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
       <c r="D6" s="4"/>
       <c r="E6" s="4"/>
       <c r="F6" s="4"/>
     </row>
-    <row r="7" ht="246.5" spans="1:6">
+    <row r="7" ht="255" spans="1:6">
       <c r="B7" s="5" t="s">
-        <v>202</v>
-      </c>
-      <c r="C7" s="18" t="s">
-        <v>250</v>
+        <v>203</v>
+      </c>
+      <c r="C7" s="19" t="s">
+        <v>251</v>
       </c>
       <c r="D7" t="s">
-        <v>251</v>
-      </c>
-      <c r="E7" s="11" t="s">
         <v>252</v>
+      </c>
+      <c r="E7" s="12" t="s">
+        <v>253</v>
       </c>
     </row>
     <row r="8" ht="71" customHeight="1" spans="1:6">
       <c r="B8" s="5" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="C8" s="4" t="s">
-        <v>254</v>
-      </c>
-      <c r="D8" s="10" t="s">
         <v>255</v>
       </c>
-      <c r="E8" s="9"/>
-    </row>
-    <row r="9" ht="29" spans="1:6">
+      <c r="D8" s="11" t="s">
+        <v>256</v>
+      </c>
+      <c r="E8" s="10"/>
+    </row>
+    <row r="9" ht="30" spans="1:6">
       <c r="B9" s="5" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
       <c r="C9" s="4" t="s">
-        <v>257</v>
-      </c>
-      <c r="D9" s="10"/>
-      <c r="E9" s="25"/>
+        <v>258</v>
+      </c>
+      <c r="D9" s="11"/>
+      <c r="E9" s="26"/>
     </row>
     <row r="10" spans="1:6">
       <c r="B10" s="5" t="s">
-        <v>258</v>
+        <v>259</v>
       </c>
       <c r="C10" s="4" t="s">
-        <v>259</v>
-      </c>
-      <c r="D10" s="10"/>
-      <c r="E10" s="9"/>
-    </row>
-    <row r="11" ht="29" spans="1:6">
+        <v>260</v>
+      </c>
+      <c r="D10" s="11"/>
+      <c r="E10" s="10"/>
+    </row>
+    <row r="11" ht="30" spans="1:6">
       <c r="B11" s="5" t="s">
-        <v>260</v>
-      </c>
-      <c r="C11" s="18" t="s">
         <v>261</v>
       </c>
-      <c r="D11" s="12" t="s">
+      <c r="C11" s="19" t="s">
         <v>262</v>
       </c>
-    </row>
-    <row r="12" ht="58" spans="1:6">
+      <c r="D11" s="13" t="s">
+        <v>263</v>
+      </c>
+    </row>
+    <row r="12" ht="60" spans="1:6">
       <c r="B12" s="5" t="s">
-        <v>263</v>
-      </c>
-      <c r="D12" s="12"/>
-      <c r="E12" s="13" t="s">
         <v>264</v>
+      </c>
+      <c r="D12" s="13"/>
+      <c r="E12" s="14" t="s">
+        <v>265</v>
       </c>
     </row>
     <row r="13" ht="33" customHeight="1" spans="1:6">
       <c r="B13" s="5" t="s">
-        <v>265</v>
+        <v>266</v>
       </c>
       <c r="C13" s="4" t="s">
-        <v>266</v>
-      </c>
-      <c r="D13" s="12"/>
+        <v>267</v>
+      </c>
+      <c r="D13" s="13"/>
     </row>
     <row r="14" customFormat="1" spans="1:6">
       <c r="B14" t="s">
-        <v>267</v>
+        <v>268</v>
       </c>
       <c r="C14" s="4" t="s">
-        <v>268</v>
-      </c>
-    </row>
-    <row r="15" customFormat="1" ht="58" spans="1:6">
+        <v>269</v>
+      </c>
+    </row>
+    <row r="15" customFormat="1" ht="60" spans="1:6">
       <c r="B15" s="5" t="s">
-        <v>269</v>
+        <v>270</v>
       </c>
       <c r="C15" t="s">
-        <v>230</v>
-      </c>
-      <c r="D15" s="10" t="s">
-        <v>270</v>
-      </c>
-    </row>
-    <row r="16" customFormat="1" ht="29" spans="1:6">
+        <v>231</v>
+      </c>
+      <c r="D15" s="11" t="s">
+        <v>271</v>
+      </c>
+    </row>
+    <row r="16" customFormat="1" ht="30" spans="1:6">
       <c r="B16" s="5" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="C16" s="4" t="s">
-        <v>272</v>
-      </c>
-    </row>
-    <row r="17" ht="58" spans="2:5">
+        <v>273</v>
+      </c>
+    </row>
+    <row r="17" ht="60" spans="2:5">
       <c r="B17" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="C17" s="4" t="s">
-        <v>274</v>
-      </c>
-      <c r="D17" s="10" t="s">
         <v>275</v>
+      </c>
+      <c r="D17" s="11" t="s">
+        <v>276</v>
       </c>
     </row>
     <row r="18" spans="2:5">
       <c r="B18" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
       <c r="C18" s="4" t="s">
-        <v>277</v>
-      </c>
-    </row>
-    <row r="19" ht="43.5" spans="2:5">
+        <v>278</v>
+      </c>
+    </row>
+    <row r="19" ht="45" spans="2:5">
       <c r="B19" t="s">
-        <v>278</v>
+        <v>279</v>
       </c>
       <c r="C19" s="4" t="s">
-        <v>279</v>
-      </c>
-      <c r="D19" s="10" t="s">
         <v>280</v>
       </c>
+      <c r="D19" s="11" t="s">
+        <v>281</v>
+      </c>
       <c r="E19" s="4" t="s">
-        <v>281</v>
+        <v>282</v>
       </c>
     </row>
     <row r="20" spans="2:5">
       <c r="B20" t="s">
-        <v>282</v>
+        <v>283</v>
       </c>
       <c r="C20" s="4" t="s">
-        <v>283</v>
-      </c>
-      <c r="E20" s="19"/>
+        <v>284</v>
+      </c>
+      <c r="E20" s="20"/>
     </row>
     <row r="21" ht="409.5" spans="2:5">
       <c r="B21" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
       <c r="C21" s="4" t="s">
-        <v>285</v>
-      </c>
-      <c r="E21" s="13" t="s">
         <v>286</v>
       </c>
-    </row>
-    <row r="22" ht="58" spans="2:5">
+      <c r="E21" s="14" t="s">
+        <v>287</v>
+      </c>
+    </row>
+    <row r="22" ht="60" spans="2:5">
       <c r="B22" t="s">
-        <v>287</v>
+        <v>288</v>
       </c>
       <c r="C22" s="4" t="s">
-        <v>288</v>
-      </c>
-      <c r="E22" s="22"/>
+        <v>289</v>
+      </c>
+      <c r="E22" s="23"/>
     </row>
     <row r="23" ht="66" customHeight="1" spans="2:5">
       <c r="B23" t="s">
-        <v>289</v>
+        <v>290</v>
       </c>
       <c r="C23" t="s">
-        <v>290</v>
-      </c>
-      <c r="D23" s="10" t="s">
         <v>291</v>
+      </c>
+      <c r="D23" s="11" t="s">
+        <v>292</v>
       </c>
       <c r="E23" s="4"/>
     </row>
     <row r="24" customFormat="1" spans="2:5">
       <c r="B24" t="s">
-        <v>292</v>
+        <v>293</v>
       </c>
       <c r="C24" s="4" t="s">
-        <v>293</v>
-      </c>
-      <c r="D24" s="10"/>
+        <v>294</v>
+      </c>
+      <c r="D24" s="11"/>
       <c r="E24" s="4"/>
     </row>
     <row r="25" customFormat="1" spans="2:5">
       <c r="B25" s="4" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="C25" s="4" t="s">
-        <v>193</v>
-      </c>
-      <c r="D25" s="14" t="s">
-        <v>294</v>
+        <v>194</v>
+      </c>
+      <c r="D25" s="15" t="s">
+        <v>295</v>
       </c>
     </row>
     <row r="26" customFormat="1" ht="46" customHeight="1" spans="2:5">
       <c r="B26" s="4" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="C26" s="4" t="s">
-        <v>295</v>
-      </c>
-      <c r="D26" s="14"/>
+        <v>296</v>
+      </c>
+      <c r="D26" s="15"/>
     </row>
   </sheetData>
   <mergeCells count="6">
@@ -9084,14 +8990,14 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
   <dimension ref="A1:F32"/>
-  <sheetFormatPr defaultColWidth="9.14545454545454" defaultRowHeight="14.5" outlineLevelCol="5"/>
+  <sheetFormatPr defaultColWidth="9.14285714285714" defaultRowHeight="15" outlineLevelCol="5"/>
   <cols>
-    <col min="1" max="1" width="14.7181818181818" customWidth="1"/>
-    <col min="2" max="2" width="27.3363636363636" customWidth="1"/>
-    <col min="3" max="3" width="50.8818181818182" customWidth="1"/>
-    <col min="4" max="4" width="72.8545454545455" customWidth="1"/>
-    <col min="5" max="5" width="46.4272727272727" customWidth="1"/>
-    <col min="6" max="6" width="45.7181818181818" customWidth="1"/>
+    <col min="1" max="1" width="14.7142857142857" customWidth="1"/>
+    <col min="2" max="2" width="27.3333333333333" customWidth="1"/>
+    <col min="3" max="3" width="50.8857142857143" customWidth="1"/>
+    <col min="4" max="4" width="72.8571428571429" customWidth="1"/>
+    <col min="5" max="5" width="46.4285714285714" customWidth="1"/>
+    <col min="6" max="6" width="45.7142857142857" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" s="1" customFormat="1" spans="1:6">
@@ -9124,15 +9030,18 @@
         <v>14</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>296</v>
-      </c>
-    </row>
-    <row r="4" spans="1:6">
+        <v>297</v>
+      </c>
+    </row>
+    <row r="4" ht="90" spans="1:6">
       <c r="B4" t="s">
         <v>16</v>
       </c>
-      <c r="C4" t="s">
-        <v>17</v>
+      <c r="C4" s="6" t="s">
+        <v>298</v>
+      </c>
+      <c r="D4" t="s">
+        <v>299</v>
       </c>
     </row>
     <row r="5" customFormat="1" spans="1:6">
@@ -9141,20 +9050,20 @@
         <v>19</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="D5" s="4"/>
       <c r="E5" s="4" t="s">
-        <v>297</v>
+        <v>300</v>
       </c>
       <c r="F5" s="4"/>
     </row>
-    <row r="6" customFormat="1" ht="29" spans="1:6">
+    <row r="6" customFormat="1" ht="30" spans="1:6">
       <c r="B6" s="4" t="s">
         <v>22</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>298</v>
+        <v>301</v>
       </c>
       <c r="D6" s="4"/>
       <c r="E6" s="4"/>
@@ -9162,294 +9071,294 @@
     </row>
     <row r="7" spans="1:6">
       <c r="B7" s="5" t="s">
-        <v>299</v>
+        <v>302</v>
       </c>
       <c r="D7" t="s">
-        <v>300</v>
-      </c>
-      <c r="E7" s="8" t="s">
-        <v>301</v>
-      </c>
-      <c r="F7" s="9" t="s">
-        <v>302</v>
+        <v>303</v>
+      </c>
+      <c r="E7" s="9" t="s">
+        <v>304</v>
+      </c>
+      <c r="F7" s="10" t="s">
+        <v>305</v>
       </c>
     </row>
     <row r="8" ht="63" customHeight="1" spans="1:6">
       <c r="B8" t="s">
-        <v>303</v>
-      </c>
-      <c r="C8" s="18" t="s">
-        <v>304</v>
-      </c>
-      <c r="D8" s="10" t="s">
-        <v>305</v>
+        <v>306</v>
+      </c>
+      <c r="C8" s="19" t="s">
+        <v>307</v>
+      </c>
+      <c r="D8" s="11" t="s">
+        <v>308</v>
       </c>
       <c r="F8" s="4" t="s">
-        <v>306</v>
+        <v>309</v>
       </c>
     </row>
     <row r="9" spans="1:6">
       <c r="B9" t="s">
-        <v>307</v>
+        <v>310</v>
       </c>
       <c r="C9" s="4" t="s">
-        <v>308</v>
-      </c>
-      <c r="D9" s="10"/>
-      <c r="E9" s="8"/>
-    </row>
-    <row r="10" ht="29" spans="1:6">
+        <v>311</v>
+      </c>
+      <c r="D9" s="11"/>
+      <c r="E9" s="9"/>
+    </row>
+    <row r="10" ht="30" spans="1:6">
       <c r="B10" s="4" t="s">
-        <v>309</v>
+        <v>312</v>
       </c>
       <c r="C10" s="4" t="s">
-        <v>310</v>
-      </c>
-      <c r="D10" s="10"/>
-      <c r="E10" s="8"/>
-    </row>
-    <row r="11" ht="29" spans="1:6">
+        <v>313</v>
+      </c>
+      <c r="D10" s="11"/>
+      <c r="E10" s="9"/>
+    </row>
+    <row r="11" ht="30" spans="1:6">
       <c r="B11" s="4" t="s">
-        <v>311</v>
+        <v>314</v>
       </c>
       <c r="C11" s="4" t="s">
-        <v>137</v>
-      </c>
-      <c r="D11" s="10"/>
-      <c r="E11" s="8"/>
-    </row>
-    <row r="12" ht="29" spans="1:6">
+        <v>138</v>
+      </c>
+      <c r="D11" s="11"/>
+      <c r="E11" s="9"/>
+    </row>
+    <row r="12" ht="30" spans="1:6">
       <c r="B12" s="4" t="s">
-        <v>312</v>
+        <v>315</v>
       </c>
       <c r="C12" s="4" t="s">
-        <v>313</v>
-      </c>
-      <c r="D12" s="10"/>
-      <c r="E12" s="8"/>
+        <v>316</v>
+      </c>
+      <c r="D12" s="11"/>
+      <c r="E12" s="9"/>
     </row>
     <row r="13" customFormat="1" ht="66" customHeight="1" spans="1:6">
       <c r="B13" t="s">
-        <v>314</v>
-      </c>
-      <c r="C13" s="18" t="s">
-        <v>315</v>
-      </c>
-      <c r="D13" s="10" t="s">
-        <v>316</v>
+        <v>317</v>
+      </c>
+      <c r="C13" s="19" t="s">
+        <v>318</v>
+      </c>
+      <c r="D13" s="11" t="s">
+        <v>319</v>
       </c>
       <c r="F13" s="4" t="s">
-        <v>306</v>
+        <v>309</v>
       </c>
     </row>
     <row r="14" customFormat="1" spans="1:6">
       <c r="B14" t="s">
-        <v>317</v>
+        <v>320</v>
       </c>
       <c r="C14" s="4" t="s">
-        <v>318</v>
-      </c>
-      <c r="D14" s="10"/>
-      <c r="E14" s="22"/>
-    </row>
-    <row r="15" customFormat="1" ht="29" spans="1:6">
+        <v>321</v>
+      </c>
+      <c r="D14" s="11"/>
+      <c r="E14" s="23"/>
+    </row>
+    <row r="15" customFormat="1" ht="30" spans="1:6">
       <c r="B15" s="4" t="s">
-        <v>319</v>
+        <v>322</v>
       </c>
       <c r="C15" s="4" t="s">
-        <v>320</v>
-      </c>
-      <c r="D15" s="10"/>
-      <c r="E15" s="22"/>
-    </row>
-    <row r="16" customFormat="1" ht="29" spans="1:6">
+        <v>323</v>
+      </c>
+      <c r="D15" s="11"/>
+      <c r="E15" s="23"/>
+    </row>
+    <row r="16" customFormat="1" ht="30" spans="1:6">
       <c r="B16" s="4" t="s">
-        <v>321</v>
+        <v>324</v>
       </c>
       <c r="C16" s="4" t="s">
-        <v>137</v>
-      </c>
-      <c r="D16" s="10"/>
+        <v>138</v>
+      </c>
+      <c r="D16" s="11"/>
       <c r="E16" s="4"/>
     </row>
-    <row r="17" customFormat="1" ht="29" spans="2:6">
+    <row r="17" customFormat="1" ht="30" spans="2:6">
       <c r="B17" s="4" t="s">
-        <v>322</v>
+        <v>325</v>
       </c>
       <c r="C17" s="4" t="s">
-        <v>323</v>
-      </c>
-      <c r="D17" s="10"/>
-    </row>
-    <row r="18" ht="29" spans="2:6">
+        <v>326</v>
+      </c>
+      <c r="D17" s="11"/>
+    </row>
+    <row r="18" ht="30" spans="2:6">
       <c r="B18" s="5" t="s">
-        <v>324</v>
-      </c>
-      <c r="C18" s="18" t="s">
-        <v>325</v>
-      </c>
-      <c r="D18" s="10" t="s">
-        <v>326</v>
+        <v>327</v>
+      </c>
+      <c r="C18" s="19" t="s">
+        <v>328</v>
+      </c>
+      <c r="D18" s="11" t="s">
+        <v>329</v>
       </c>
       <c r="E18" s="4"/>
     </row>
     <row r="19" ht="93" customHeight="1" spans="2:6">
       <c r="B19" t="s">
-        <v>327</v>
-      </c>
-      <c r="D19" s="10" t="s">
-        <v>328</v>
-      </c>
-      <c r="F19" s="8" t="s">
-        <v>329</v>
+        <v>330</v>
+      </c>
+      <c r="D19" s="11" t="s">
+        <v>331</v>
+      </c>
+      <c r="F19" s="9" t="s">
+        <v>332</v>
       </c>
     </row>
     <row r="20" customFormat="1" spans="2:6">
       <c r="B20" t="s">
-        <v>330</v>
+        <v>333</v>
       </c>
       <c r="C20" s="4"/>
-      <c r="D20" s="10"/>
-      <c r="F20" s="8" t="s">
-        <v>331</v>
-      </c>
-    </row>
-    <row r="21" customFormat="1" ht="116" spans="2:6">
+      <c r="D20" s="11"/>
+      <c r="F20" s="9" t="s">
+        <v>334</v>
+      </c>
+    </row>
+    <row r="21" customFormat="1" ht="120" spans="2:6">
       <c r="B21" s="4" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="C21" s="4"/>
-      <c r="D21" s="10" t="s">
-        <v>332</v>
-      </c>
-      <c r="E21" s="18" t="s">
-        <v>102</v>
+      <c r="D21" s="11" t="s">
+        <v>335</v>
+      </c>
+      <c r="E21" s="19" t="s">
+        <v>103</v>
       </c>
       <c r="F21" s="4"/>
     </row>
-    <row r="22" customFormat="1" ht="29" spans="2:6">
+    <row r="22" customFormat="1" ht="30" spans="2:6">
       <c r="B22" s="4" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="C22" s="4" t="s">
-        <v>333</v>
-      </c>
-      <c r="D22" s="10"/>
+        <v>336</v>
+      </c>
+      <c r="D22" s="11"/>
       <c r="F22" s="4"/>
     </row>
-    <row r="23" customFormat="1" ht="87" spans="2:6">
+    <row r="23" customFormat="1" ht="90" spans="2:6">
       <c r="B23" s="4" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="C23" s="4" t="s">
-        <v>334</v>
-      </c>
-      <c r="D23" s="10"/>
-      <c r="E23" s="23" t="s">
-        <v>335</v>
+        <v>337</v>
+      </c>
+      <c r="D23" s="11"/>
+      <c r="E23" s="24" t="s">
+        <v>338</v>
       </c>
       <c r="F23" s="4"/>
     </row>
-    <row r="24" customFormat="1" ht="116" spans="2:6">
+    <row r="24" customFormat="1" ht="120" spans="2:6">
       <c r="B24" s="4" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="C24" s="4" t="s">
-        <v>336</v>
-      </c>
-      <c r="D24" s="10" t="s">
-        <v>337</v>
+        <v>339</v>
+      </c>
+      <c r="D24" s="11" t="s">
+        <v>340</v>
       </c>
       <c r="E24" s="4"/>
       <c r="F24" s="4"/>
     </row>
-    <row r="25" customFormat="1" ht="72.5" spans="2:6">
+    <row r="25" customFormat="1" ht="75" spans="2:6">
       <c r="B25" s="4" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="C25" s="4" t="s">
-        <v>338</v>
-      </c>
-      <c r="D25" s="10"/>
-      <c r="E25" s="13" t="s">
-        <v>339</v>
+        <v>341</v>
+      </c>
+      <c r="D25" s="11"/>
+      <c r="E25" s="14" t="s">
+        <v>342</v>
       </c>
       <c r="F25" s="4"/>
     </row>
-    <row r="26" customFormat="1" ht="29" spans="2:6">
+    <row r="26" customFormat="1" ht="30" spans="2:6">
       <c r="B26" s="4" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="C26" s="4" t="s">
-        <v>340</v>
-      </c>
-      <c r="D26" s="10"/>
+        <v>343</v>
+      </c>
+      <c r="D26" s="11"/>
       <c r="E26" s="4"/>
       <c r="F26" s="4"/>
     </row>
-    <row r="27" customFormat="1" ht="29" spans="2:6">
+    <row r="27" customFormat="1" ht="30" spans="2:6">
       <c r="B27" s="4" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="C27" s="4" t="s">
-        <v>341</v>
-      </c>
-      <c r="D27" s="10"/>
+        <v>344</v>
+      </c>
+      <c r="D27" s="11"/>
       <c r="E27" s="4"/>
       <c r="F27" s="4"/>
     </row>
-    <row r="28" customFormat="1" ht="29" spans="2:6">
+    <row r="28" customFormat="1" ht="30" spans="2:6">
       <c r="B28" s="4" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="C28" s="4" t="s">
-        <v>342</v>
-      </c>
-      <c r="D28" s="10"/>
+        <v>345</v>
+      </c>
+      <c r="D28" s="11"/>
       <c r="E28" s="4"/>
       <c r="F28" s="4"/>
     </row>
-    <row r="29" customFormat="1" ht="29" spans="2:6">
+    <row r="29" customFormat="1" ht="30" spans="2:6">
       <c r="B29" s="4" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="C29" s="4" t="s">
-        <v>343</v>
-      </c>
-      <c r="D29" s="10"/>
+        <v>346</v>
+      </c>
+      <c r="D29" s="11"/>
       <c r="E29" s="4"/>
       <c r="F29" s="4"/>
     </row>
-    <row r="30" customFormat="1" ht="29" spans="2:6">
+    <row r="30" customFormat="1" ht="30" spans="2:6">
       <c r="B30" s="4" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="C30" s="4" t="s">
-        <v>344</v>
-      </c>
-      <c r="D30" s="10"/>
+        <v>347</v>
+      </c>
+      <c r="D30" s="11"/>
       <c r="E30" s="4"/>
       <c r="F30" s="4"/>
     </row>
     <row r="31" customFormat="1" spans="2:6">
       <c r="B31" s="4" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="C31" s="4" t="s">
-        <v>193</v>
-      </c>
-      <c r="D31" s="14" t="s">
-        <v>345</v>
+        <v>194</v>
+      </c>
+      <c r="D31" s="15" t="s">
+        <v>348</v>
       </c>
     </row>
     <row r="32" customFormat="1" ht="46" customHeight="1" spans="2:6">
       <c r="B32" s="4" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="C32" s="4" t="s">
-        <v>346</v>
-      </c>
-      <c r="D32" s="14"/>
+        <v>349</v>
+      </c>
+      <c r="D32" s="15"/>
     </row>
   </sheetData>
   <mergeCells count="6">
@@ -9469,13 +9378,13 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
   <dimension ref="A1:F21"/>
-  <sheetFormatPr defaultColWidth="8.88181818181818" defaultRowHeight="14.5" outlineLevelCol="5"/>
+  <sheetFormatPr defaultColWidth="8.88571428571429" defaultRowHeight="15" outlineLevelCol="5"/>
   <cols>
-    <col min="1" max="1" width="14.7181818181818" customWidth="1"/>
-    <col min="2" max="2" width="33.8818181818182" customWidth="1"/>
-    <col min="3" max="3" width="46.8545454545455" customWidth="1"/>
-    <col min="4" max="4" width="57.1181818181818" customWidth="1"/>
-    <col min="5" max="5" width="54.7181818181818" customWidth="1"/>
+    <col min="1" max="1" width="14.7142857142857" customWidth="1"/>
+    <col min="2" max="2" width="33.8857142857143" customWidth="1"/>
+    <col min="3" max="3" width="62.5714285714286" customWidth="1"/>
+    <col min="4" max="4" width="57.1142857142857" customWidth="1"/>
+    <col min="5" max="5" width="54.7142857142857" customWidth="1"/>
     <col min="6" max="6" width="38" customWidth="1"/>
   </cols>
   <sheetData>
@@ -9499,9 +9408,9 @@
         <v>50</v>
       </c>
     </row>
-    <row r="2" ht="43.5" spans="1:6">
-      <c r="A2" s="21" t="s">
-        <v>347</v>
+    <row r="2" ht="45" spans="1:6">
+      <c r="A2" s="22" t="s">
+        <v>350</v>
       </c>
     </row>
     <row r="3" spans="1:6">
@@ -9510,39 +9419,39 @@
         <v>14</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>348</v>
-      </c>
-    </row>
-    <row r="4" spans="1:6">
+        <v>351</v>
+      </c>
+    </row>
+    <row r="4" ht="240" spans="1:6">
       <c r="A4" s="1"/>
       <c r="B4" s="5" t="s">
         <v>16</v>
       </c>
-      <c r="C4" t="s">
-        <v>17</v>
+      <c r="C4" s="6" t="s">
+        <v>352</v>
       </c>
       <c r="D4" t="s">
-        <v>349</v>
+        <v>353</v>
       </c>
     </row>
     <row r="5" spans="1:6">
       <c r="A5" s="1"/>
-      <c r="B5" s="15" t="s">
+      <c r="B5" s="16" t="s">
         <v>19</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="D5" s="4"/>
       <c r="E5" s="4"/>
       <c r="F5" s="4"/>
     </row>
-    <row r="6" ht="29" spans="1:6">
-      <c r="B6" s="15" t="s">
+    <row r="6" ht="30" spans="1:6">
+      <c r="B6" s="16" t="s">
         <v>22</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>350</v>
+        <v>354</v>
       </c>
       <c r="D6" s="4"/>
       <c r="E6" s="4"/>
@@ -9550,163 +9459,163 @@
     </row>
     <row r="7" spans="1:6">
       <c r="B7" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="D7" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="F7" s="4" t="s">
-        <v>351</v>
-      </c>
-    </row>
-    <row r="8" ht="145" spans="1:6">
+        <v>355</v>
+      </c>
+    </row>
+    <row r="8" ht="150" spans="1:6">
       <c r="B8" s="5" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="C8" s="4" t="s">
-        <v>352</v>
+        <v>356</v>
       </c>
       <c r="D8" t="s">
-        <v>353</v>
-      </c>
-      <c r="E8" s="11" t="s">
-        <v>354</v>
+        <v>357</v>
+      </c>
+      <c r="E8" s="12" t="s">
+        <v>358</v>
       </c>
     </row>
     <row r="9" ht="70" customHeight="1" spans="1:6">
       <c r="B9" s="5" t="s">
-        <v>355</v>
+        <v>359</v>
       </c>
       <c r="C9" s="4" t="s">
-        <v>356</v>
-      </c>
-      <c r="D9" s="10" t="s">
-        <v>357</v>
-      </c>
-    </row>
-    <row r="10" ht="29" spans="1:6">
+        <v>360</v>
+      </c>
+      <c r="D9" s="11" t="s">
+        <v>361</v>
+      </c>
+    </row>
+    <row r="10" ht="30" spans="1:6">
       <c r="B10" s="5" t="s">
-        <v>358</v>
+        <v>362</v>
       </c>
       <c r="C10" s="4" t="s">
-        <v>359</v>
-      </c>
-      <c r="D10" s="10"/>
+        <v>363</v>
+      </c>
+      <c r="D10" s="11"/>
     </row>
     <row r="11" spans="1:6">
       <c r="B11" s="5" t="s">
-        <v>360</v>
+        <v>364</v>
       </c>
       <c r="C11" s="4" t="s">
-        <v>220</v>
-      </c>
-      <c r="D11" s="10"/>
-      <c r="E11" s="8"/>
-    </row>
-    <row r="12" ht="29" spans="1:6">
+        <v>221</v>
+      </c>
+      <c r="D11" s="11"/>
+      <c r="E11" s="9"/>
+    </row>
+    <row r="12" ht="30" spans="1:6">
       <c r="B12" s="5" t="s">
-        <v>361</v>
+        <v>365</v>
       </c>
       <c r="C12" s="4" t="s">
-        <v>359</v>
-      </c>
-      <c r="D12" s="10"/>
+        <v>363</v>
+      </c>
+      <c r="D12" s="11"/>
     </row>
     <row r="13" ht="38" customHeight="1" spans="1:6">
       <c r="B13" s="4" t="s">
-        <v>362</v>
+        <v>366</v>
       </c>
       <c r="C13" s="4" t="s">
-        <v>363</v>
-      </c>
-      <c r="D13" s="10" t="s">
-        <v>364</v>
-      </c>
-    </row>
-    <row r="14" ht="29" spans="1:6">
+        <v>367</v>
+      </c>
+      <c r="D13" s="11" t="s">
+        <v>368</v>
+      </c>
+    </row>
+    <row r="14" ht="30" spans="1:6">
       <c r="B14" s="4" t="s">
-        <v>365</v>
+        <v>369</v>
       </c>
       <c r="C14" s="4" t="s">
-        <v>366</v>
-      </c>
-      <c r="D14" s="10"/>
+        <v>370</v>
+      </c>
+      <c r="D14" s="11"/>
     </row>
     <row r="15" ht="153" customHeight="1" spans="1:6">
       <c r="B15" s="4" t="s">
-        <v>367</v>
+        <v>371</v>
       </c>
       <c r="C15" s="4" t="s">
-        <v>368</v>
-      </c>
-      <c r="D15" s="10"/>
-      <c r="E15" s="8" t="s">
-        <v>369</v>
-      </c>
-    </row>
-    <row r="16" ht="58" spans="1:6">
+        <v>372</v>
+      </c>
+      <c r="D15" s="11"/>
+      <c r="E15" s="9" t="s">
+        <v>373</v>
+      </c>
+    </row>
+    <row r="16" ht="75" spans="1:6">
       <c r="B16" s="5" t="s">
-        <v>269</v>
+        <v>270</v>
       </c>
       <c r="C16" t="s">
-        <v>230</v>
-      </c>
-      <c r="D16" s="10" t="s">
-        <v>270</v>
-      </c>
-    </row>
-    <row r="17" ht="29" spans="2:6">
+        <v>231</v>
+      </c>
+      <c r="D16" s="11" t="s">
+        <v>271</v>
+      </c>
+    </row>
+    <row r="17" ht="30" spans="2:6">
       <c r="B17" s="5" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="C17" s="4" t="s">
-        <v>272</v>
-      </c>
-    </row>
-    <row r="18" ht="87" spans="2:6">
+        <v>273</v>
+      </c>
+    </row>
+    <row r="18" ht="90" spans="2:6">
       <c r="B18" t="s">
-        <v>370</v>
+        <v>374</v>
       </c>
       <c r="C18" s="4" t="s">
-        <v>371</v>
+        <v>375</v>
       </c>
       <c r="D18" t="s">
-        <v>372</v>
+        <v>376</v>
       </c>
       <c r="E18" s="4" t="s">
-        <v>373</v>
+        <v>377</v>
       </c>
     </row>
     <row r="19" spans="2:6">
       <c r="B19" t="s">
-        <v>374</v>
+        <v>378</v>
       </c>
       <c r="D19" t="s">
-        <v>375</v>
-      </c>
-      <c r="F19" s="19" t="s">
-        <v>376</v>
+        <v>379</v>
+      </c>
+      <c r="F19" s="20" t="s">
+        <v>380</v>
       </c>
     </row>
     <row r="20" spans="2:6">
       <c r="B20" s="4" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="C20" s="4" t="s">
-        <v>193</v>
-      </c>
-      <c r="D20" s="14" t="s">
-        <v>377</v>
+        <v>194</v>
+      </c>
+      <c r="D20" s="15" t="s">
+        <v>381</v>
       </c>
     </row>
     <row r="21" ht="45" customHeight="1" spans="2:6">
       <c r="B21" s="4" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="C21" s="4" t="s">
-        <v>378</v>
-      </c>
-      <c r="D21" s="14"/>
+        <v>382</v>
+      </c>
+      <c r="D21" s="15"/>
     </row>
   </sheetData>
   <mergeCells count="3">
@@ -9723,14 +9632,14 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
   <dimension ref="A1:F31"/>
-  <sheetFormatPr defaultColWidth="9.14545454545454" defaultRowHeight="14.5" outlineLevelCol="5"/>
+  <sheetFormatPr defaultColWidth="9.14285714285714" defaultRowHeight="15" outlineLevelCol="5"/>
   <cols>
-    <col min="1" max="1" width="14.7181818181818" customWidth="1"/>
-    <col min="2" max="2" width="34.5727272727273" customWidth="1"/>
-    <col min="3" max="3" width="49.6636363636364" customWidth="1"/>
-    <col min="4" max="4" width="56.5545454545455" customWidth="1"/>
-    <col min="5" max="5" width="53.2818181818182" customWidth="1"/>
-    <col min="6" max="6" width="50.2818181818182" customWidth="1"/>
+    <col min="1" max="1" width="14.7142857142857" customWidth="1"/>
+    <col min="2" max="2" width="34.5714285714286" customWidth="1"/>
+    <col min="3" max="3" width="49.6666666666667" customWidth="1"/>
+    <col min="4" max="4" width="58.4285714285714" customWidth="1"/>
+    <col min="5" max="5" width="53.2857142857143" customWidth="1"/>
+    <col min="6" max="6" width="50.2857142857143" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" s="1" customFormat="1" spans="1:6">
@@ -9758,12 +9667,12 @@
         <v>44</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>379</v>
+        <v>383</v>
       </c>
       <c r="C2" s="3"/>
       <c r="D2" s="3"/>
       <c r="E2" s="3"/>
-      <c r="F2" s="20"/>
+      <c r="F2" s="21"/>
     </row>
     <row r="3" spans="1:6">
       <c r="A3" s="1"/>
@@ -9771,40 +9680,40 @@
         <v>14</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>348</v>
-      </c>
-    </row>
-    <row r="4" ht="82.5" spans="1:6">
+        <v>351</v>
+      </c>
+    </row>
+    <row r="4" ht="90" spans="1:6">
       <c r="A4" s="1"/>
       <c r="B4" s="5" t="s">
         <v>16</v>
       </c>
-      <c r="C4" s="18" t="s">
-        <v>380</v>
+      <c r="C4" s="19" t="s">
+        <v>384</v>
       </c>
       <c r="D4" s="4" t="s">
-        <v>381</v>
-      </c>
-      <c r="E4" s="18"/>
+        <v>385</v>
+      </c>
+      <c r="E4" s="19"/>
     </row>
     <row r="5" customFormat="1" spans="1:6">
       <c r="A5" s="1"/>
-      <c r="B5" s="15" t="s">
+      <c r="B5" s="16" t="s">
         <v>19</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="D5" s="4"/>
       <c r="E5" s="4"/>
       <c r="F5" s="4"/>
     </row>
-    <row r="6" customFormat="1" ht="29" spans="1:6">
-      <c r="B6" s="15" t="s">
+    <row r="6" customFormat="1" ht="30" spans="1:6">
+      <c r="B6" s="16" t="s">
         <v>22</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>382</v>
+        <v>386</v>
       </c>
       <c r="D6" s="4"/>
       <c r="E6" s="4"/>
@@ -9812,272 +9721,272 @@
     </row>
     <row r="7" spans="1:6">
       <c r="B7" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="D7" t="s">
-        <v>57</v>
-      </c>
-      <c r="F7" s="8" t="s">
-        <v>351</v>
-      </c>
-    </row>
-    <row r="8" ht="101.5" spans="1:6">
+        <v>58</v>
+      </c>
+      <c r="F7" s="9" t="s">
+        <v>355</v>
+      </c>
+    </row>
+    <row r="8" ht="105" spans="1:6">
       <c r="B8" s="5" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="C8" s="4" t="s">
-        <v>383</v>
+        <v>387</v>
       </c>
       <c r="D8" t="s">
-        <v>353</v>
-      </c>
-      <c r="E8" s="16" t="s">
-        <v>384</v>
+        <v>357</v>
+      </c>
+      <c r="E8" s="17" t="s">
+        <v>388</v>
       </c>
     </row>
     <row r="9" ht="139" customHeight="1" spans="1:6">
       <c r="B9" s="5" t="s">
-        <v>385</v>
-      </c>
-      <c r="D9" s="6" t="s">
-        <v>386</v>
-      </c>
-      <c r="E9" s="18" t="s">
-        <v>387</v>
-      </c>
-    </row>
-    <row r="10" ht="43.5" spans="1:6">
+        <v>389</v>
+      </c>
+      <c r="D9" s="7" t="s">
+        <v>390</v>
+      </c>
+      <c r="E9" s="19" t="s">
+        <v>391</v>
+      </c>
+    </row>
+    <row r="10" ht="45" spans="1:6">
       <c r="B10" s="5" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
       <c r="C10" s="4" t="s">
-        <v>388</v>
-      </c>
-      <c r="D10" s="6"/>
-      <c r="E10" s="8" t="s">
-        <v>389</v>
-      </c>
-    </row>
-    <row r="11" ht="203" spans="1:6">
+        <v>392</v>
+      </c>
+      <c r="D10" s="7"/>
+      <c r="E10" s="9" t="s">
+        <v>393</v>
+      </c>
+    </row>
+    <row r="11" ht="210" spans="1:6">
       <c r="B11" s="5" t="s">
-        <v>214</v>
-      </c>
-      <c r="D11" s="6"/>
-      <c r="E11" s="11" t="s">
-        <v>390</v>
-      </c>
-    </row>
-    <row r="12" ht="203" spans="1:6">
+        <v>215</v>
+      </c>
+      <c r="D11" s="7"/>
+      <c r="E11" s="12" t="s">
+        <v>394</v>
+      </c>
+    </row>
+    <row r="12" ht="210" spans="1:6">
       <c r="B12" s="5" t="s">
-        <v>217</v>
-      </c>
-      <c r="D12" s="6"/>
-      <c r="E12" s="11" t="s">
-        <v>391</v>
+        <v>218</v>
+      </c>
+      <c r="D12" s="7"/>
+      <c r="E12" s="12" t="s">
+        <v>395</v>
       </c>
     </row>
     <row r="13" spans="1:6">
       <c r="B13" s="5" t="s">
-        <v>392</v>
-      </c>
-      <c r="D13" s="6"/>
-      <c r="E13" s="8" t="s">
-        <v>393</v>
+        <v>396</v>
+      </c>
+      <c r="D13" s="7"/>
+      <c r="E13" s="9" t="s">
+        <v>397</v>
       </c>
     </row>
     <row r="14" ht="84" customHeight="1" spans="1:6">
       <c r="B14" s="5" t="s">
-        <v>355</v>
-      </c>
-      <c r="C14" s="18" t="s">
-        <v>394</v>
-      </c>
-      <c r="D14" s="10" t="s">
-        <v>357</v>
-      </c>
-      <c r="E14" s="18" t="s">
-        <v>395</v>
+        <v>359</v>
+      </c>
+      <c r="C14" s="19" t="s">
+        <v>398</v>
+      </c>
+      <c r="D14" s="11" t="s">
+        <v>361</v>
+      </c>
+      <c r="E14" s="19" t="s">
+        <v>399</v>
       </c>
     </row>
     <row r="15" spans="1:6">
       <c r="B15" s="5" t="s">
-        <v>358</v>
+        <v>362</v>
       </c>
       <c r="C15" s="4" t="s">
-        <v>259</v>
-      </c>
-      <c r="D15" s="10"/>
-      <c r="E15" s="9"/>
+        <v>260</v>
+      </c>
+      <c r="D15" s="11"/>
+      <c r="E15" s="10"/>
     </row>
     <row r="16" spans="1:6">
       <c r="B16" s="5" t="s">
-        <v>360</v>
+        <v>364</v>
       </c>
       <c r="C16" s="4" t="s">
-        <v>220</v>
-      </c>
-      <c r="D16" s="10"/>
-      <c r="E16" s="9"/>
-    </row>
-    <row r="17" ht="29" spans="2:6">
+        <v>221</v>
+      </c>
+      <c r="D16" s="11"/>
+      <c r="E16" s="10"/>
+    </row>
+    <row r="17" ht="30" spans="2:6">
       <c r="B17" s="5" t="s">
-        <v>361</v>
+        <v>365</v>
       </c>
       <c r="C17" s="4" t="s">
-        <v>396</v>
-      </c>
-      <c r="D17" s="10"/>
-      <c r="E17" s="8" t="s">
-        <v>397</v>
-      </c>
-    </row>
-    <row r="18" ht="101.5" spans="2:6">
+        <v>400</v>
+      </c>
+      <c r="D17" s="11"/>
+      <c r="E17" s="9" t="s">
+        <v>401</v>
+      </c>
+    </row>
+    <row r="18" ht="105" spans="2:6">
       <c r="B18" s="4" t="s">
-        <v>362</v>
+        <v>366</v>
       </c>
       <c r="C18" s="4" t="s">
-        <v>398</v>
-      </c>
-      <c r="D18" s="10" t="s">
-        <v>399</v>
-      </c>
-      <c r="E18" s="18" t="s">
-        <v>400</v>
-      </c>
-    </row>
-    <row r="19" ht="29" spans="2:6">
+        <v>402</v>
+      </c>
+      <c r="D18" s="11" t="s">
+        <v>403</v>
+      </c>
+      <c r="E18" s="19" t="s">
+        <v>404</v>
+      </c>
+    </row>
+    <row r="19" ht="30" spans="2:6">
       <c r="B19" s="4" t="s">
-        <v>365</v>
+        <v>369</v>
       </c>
       <c r="C19" s="4" t="s">
-        <v>401</v>
-      </c>
-    </row>
-    <row r="20" ht="29" spans="2:6">
+        <v>405</v>
+      </c>
+    </row>
+    <row r="20" ht="30" spans="2:6">
       <c r="B20" s="4" t="s">
-        <v>367</v>
+        <v>371</v>
       </c>
       <c r="C20" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
     </row>
     <row r="21" ht="37" customHeight="1" spans="2:6">
       <c r="B21" s="5" t="s">
-        <v>402</v>
+        <v>406</v>
       </c>
       <c r="C21" s="4" t="s">
-        <v>403</v>
-      </c>
-      <c r="D21" s="12" t="s">
-        <v>404</v>
-      </c>
-      <c r="E21" s="8"/>
-    </row>
-    <row r="22" ht="72.5" spans="2:6">
+        <v>407</v>
+      </c>
+      <c r="D21" s="13" t="s">
+        <v>408</v>
+      </c>
+      <c r="E21" s="9"/>
+    </row>
+    <row r="22" ht="75" spans="2:6">
       <c r="B22" s="5" t="s">
-        <v>405</v>
+        <v>409</v>
       </c>
       <c r="C22" t="s">
-        <v>406</v>
-      </c>
-      <c r="D22" s="12"/>
-      <c r="E22" s="11" t="s">
-        <v>407</v>
-      </c>
-    </row>
-    <row r="23" ht="43.5" spans="2:6">
+        <v>410</v>
+      </c>
+      <c r="D22" s="13"/>
+      <c r="E22" s="12" t="s">
+        <v>411</v>
+      </c>
+    </row>
+    <row r="23" ht="45" spans="2:6">
       <c r="B23" s="5" t="s">
-        <v>408</v>
-      </c>
-      <c r="D23" s="12"/>
-      <c r="E23" s="11" t="s">
-        <v>409</v>
-      </c>
-    </row>
-    <row r="24" ht="58" spans="2:6">
+        <v>412</v>
+      </c>
+      <c r="D23" s="13"/>
+      <c r="E23" s="12" t="s">
+        <v>413</v>
+      </c>
+    </row>
+    <row r="24" ht="75" spans="2:6">
       <c r="B24" s="5" t="s">
-        <v>269</v>
+        <v>270</v>
       </c>
       <c r="C24" t="s">
-        <v>230</v>
-      </c>
-      <c r="D24" s="10" t="s">
-        <v>270</v>
-      </c>
-    </row>
-    <row r="25" ht="29" spans="2:6">
+        <v>231</v>
+      </c>
+      <c r="D24" s="11" t="s">
+        <v>271</v>
+      </c>
+    </row>
+    <row r="25" ht="30" spans="2:6">
       <c r="B25" s="5" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="C25" s="4" t="s">
-        <v>272</v>
-      </c>
-    </row>
-    <row r="26" ht="43.5" spans="2:6">
+        <v>273</v>
+      </c>
+    </row>
+    <row r="26" ht="45" spans="2:6">
       <c r="B26" s="5" t="s">
-        <v>410</v>
+        <v>414</v>
       </c>
       <c r="C26" t="s">
-        <v>411</v>
+        <v>415</v>
       </c>
       <c r="D26" s="4" t="s">
-        <v>412</v>
-      </c>
-    </row>
-    <row r="27" ht="203" spans="2:6">
+        <v>416</v>
+      </c>
+    </row>
+    <row r="27" ht="210" spans="2:6">
       <c r="B27" s="5" t="s">
-        <v>370</v>
+        <v>374</v>
       </c>
       <c r="C27" s="4"/>
       <c r="D27" t="s">
-        <v>372</v>
-      </c>
-      <c r="E27" s="18" t="s">
-        <v>413</v>
-      </c>
-    </row>
-    <row r="28" ht="43.5" spans="2:6">
+        <v>376</v>
+      </c>
+      <c r="E27" s="19" t="s">
+        <v>417</v>
+      </c>
+    </row>
+    <row r="28" ht="45" spans="2:6">
       <c r="B28" s="5" t="s">
-        <v>414</v>
+        <v>418</v>
       </c>
       <c r="C28" s="4" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="D28" s="4" t="s">
-        <v>415</v>
+        <v>419</v>
       </c>
     </row>
     <row r="29" spans="2:6">
       <c r="B29" t="s">
-        <v>374</v>
+        <v>378</v>
       </c>
       <c r="D29" t="s">
-        <v>375</v>
-      </c>
-      <c r="E29" s="8"/>
-      <c r="F29" s="8" t="s">
-        <v>376</v>
+        <v>379</v>
+      </c>
+      <c r="E29" s="9"/>
+      <c r="F29" s="9" t="s">
+        <v>380</v>
       </c>
     </row>
     <row r="30" spans="2:6">
       <c r="B30" s="4" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="C30" s="4" t="s">
-        <v>193</v>
-      </c>
-      <c r="D30" s="14" t="s">
-        <v>416</v>
+        <v>194</v>
+      </c>
+      <c r="D30" s="15" t="s">
+        <v>420</v>
       </c>
     </row>
     <row r="31" ht="46" customHeight="1" spans="2:6">
       <c r="B31" s="4" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="C31" s="4" t="s">
-        <v>378</v>
-      </c>
-      <c r="D31" s="14"/>
+        <v>382</v>
+      </c>
+      <c r="D31" s="15"/>
     </row>
   </sheetData>
   <mergeCells count="5">
@@ -10096,14 +10005,14 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
   <dimension ref="A1:F21"/>
-  <sheetFormatPr defaultColWidth="9.14545454545454" defaultRowHeight="14.5" outlineLevelCol="5"/>
+  <sheetFormatPr defaultColWidth="9.14285714285714" defaultRowHeight="15" outlineLevelCol="5"/>
   <cols>
-    <col min="1" max="1" width="14.7181818181818" customWidth="1"/>
-    <col min="2" max="2" width="33.5727272727273" customWidth="1"/>
-    <col min="3" max="3" width="49.6636363636364" customWidth="1"/>
-    <col min="4" max="4" width="56.5545454545455" customWidth="1"/>
-    <col min="5" max="5" width="53.2818181818182" customWidth="1"/>
-    <col min="6" max="6" width="47.5727272727273" customWidth="1"/>
+    <col min="1" max="1" width="14.7142857142857" customWidth="1"/>
+    <col min="2" max="2" width="33.5714285714286" customWidth="1"/>
+    <col min="3" max="3" width="63.2857142857143" customWidth="1"/>
+    <col min="4" max="4" width="56.552380952381" customWidth="1"/>
+    <col min="5" max="5" width="53.2857142857143" customWidth="1"/>
+    <col min="6" max="6" width="47.5714285714286" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" s="1" customFormat="1" spans="1:6">
@@ -10131,7 +10040,7 @@
         <v>44</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>417</v>
+        <v>421</v>
       </c>
       <c r="C2" s="3"/>
       <c r="D2" s="3"/>
@@ -10144,39 +10053,39 @@
         <v>14</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>348</v>
-      </c>
-    </row>
-    <row r="4" spans="1:6">
+        <v>351</v>
+      </c>
+    </row>
+    <row r="4" ht="180" spans="1:6">
       <c r="A4" s="1"/>
       <c r="B4" s="5" t="s">
         <v>16</v>
       </c>
-      <c r="C4" t="s">
-        <v>17</v>
+      <c r="C4" s="6" t="s">
+        <v>422</v>
       </c>
       <c r="D4" t="s">
-        <v>418</v>
+        <v>423</v>
       </c>
     </row>
     <row r="5" customFormat="1" spans="1:6">
       <c r="A5" s="1"/>
-      <c r="B5" s="15" t="s">
+      <c r="B5" s="16" t="s">
         <v>19</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="D5" s="4"/>
       <c r="E5" s="4"/>
       <c r="F5" s="4"/>
     </row>
-    <row r="6" customFormat="1" ht="29" spans="1:6">
-      <c r="B6" s="15" t="s">
+    <row r="6" customFormat="1" ht="30" spans="1:6">
+      <c r="B6" s="16" t="s">
         <v>22</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>382</v>
+        <v>386</v>
       </c>
       <c r="D6" s="4"/>
       <c r="E6" s="4"/>
@@ -10184,173 +10093,173 @@
     </row>
     <row r="7" spans="1:6">
       <c r="B7" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="D7" t="s">
-        <v>57</v>
-      </c>
-      <c r="E7" s="8" t="s">
-        <v>419</v>
-      </c>
-      <c r="F7" s="8" t="s">
-        <v>351</v>
-      </c>
-    </row>
-    <row r="8" ht="101.5" spans="1:6">
+        <v>58</v>
+      </c>
+      <c r="E7" s="9" t="s">
+        <v>424</v>
+      </c>
+      <c r="F7" s="9" t="s">
+        <v>355</v>
+      </c>
+    </row>
+    <row r="8" ht="105" spans="1:6">
       <c r="B8" s="5" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="C8" s="4" t="s">
-        <v>383</v>
+        <v>387</v>
       </c>
       <c r="D8" t="s">
-        <v>353</v>
-      </c>
-      <c r="E8" s="16" t="s">
-        <v>384</v>
-      </c>
-      <c r="F8" s="17"/>
+        <v>357</v>
+      </c>
+      <c r="E8" s="17" t="s">
+        <v>388</v>
+      </c>
+      <c r="F8" s="18"/>
     </row>
     <row r="9" ht="409" customHeight="1" spans="1:6">
       <c r="B9" s="5" t="s">
-        <v>385</v>
-      </c>
-      <c r="D9" s="10" t="s">
-        <v>420</v>
+        <v>389</v>
+      </c>
+      <c r="D9" s="11" t="s">
+        <v>425</v>
       </c>
       <c r="E9" s="4" t="s">
-        <v>421</v>
-      </c>
-    </row>
-    <row r="10" ht="159.5" spans="1:6">
+        <v>426</v>
+      </c>
+    </row>
+    <row r="10" ht="165" spans="1:6">
       <c r="B10" s="5" t="s">
-        <v>355</v>
+        <v>359</v>
       </c>
       <c r="C10" s="4" t="s">
-        <v>254</v>
-      </c>
-      <c r="D10" s="10" t="s">
-        <v>422</v>
-      </c>
-      <c r="E10" s="18" t="s">
-        <v>423</v>
-      </c>
-    </row>
-    <row r="11" ht="159.5" spans="1:6">
+        <v>255</v>
+      </c>
+      <c r="D10" s="11" t="s">
+        <v>427</v>
+      </c>
+      <c r="E10" s="19" t="s">
+        <v>428</v>
+      </c>
+    </row>
+    <row r="11" ht="180" spans="1:6">
       <c r="B11" s="5" t="s">
-        <v>358</v>
+        <v>362</v>
       </c>
       <c r="C11" s="4"/>
-      <c r="E11" s="11" t="s">
-        <v>424</v>
-      </c>
-    </row>
-    <row r="12" ht="145" spans="1:6">
+      <c r="E11" s="12" t="s">
+        <v>429</v>
+      </c>
+    </row>
+    <row r="12" ht="150" spans="1:6">
       <c r="B12" s="5" t="s">
-        <v>360</v>
+        <v>364</v>
       </c>
       <c r="C12" s="4"/>
-      <c r="E12" s="11" t="s">
-        <v>425</v>
-      </c>
-    </row>
-    <row r="13" ht="58" spans="1:6">
+      <c r="E12" s="12" t="s">
+        <v>430</v>
+      </c>
+    </row>
+    <row r="13" ht="75" spans="1:6">
       <c r="B13" s="5" t="s">
-        <v>269</v>
+        <v>270</v>
       </c>
       <c r="C13" t="s">
-        <v>230</v>
-      </c>
-      <c r="D13" s="10" t="s">
-        <v>270</v>
-      </c>
-    </row>
-    <row r="14" ht="29" spans="1:6">
+        <v>231</v>
+      </c>
+      <c r="D13" s="11" t="s">
+        <v>271</v>
+      </c>
+    </row>
+    <row r="14" ht="30" spans="1:6">
       <c r="B14" s="5" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="C14" s="4" t="s">
-        <v>272</v>
-      </c>
-    </row>
-    <row r="15" ht="43.5" spans="1:6">
+        <v>273</v>
+      </c>
+    </row>
+    <row r="15" ht="45" spans="1:6">
       <c r="B15" s="5" t="s">
-        <v>410</v>
+        <v>414</v>
       </c>
       <c r="C15" t="s">
-        <v>411</v>
+        <v>415</v>
       </c>
       <c r="D15" s="4" t="s">
-        <v>412</v>
-      </c>
-    </row>
-    <row r="16" ht="203" spans="1:6">
+        <v>416</v>
+      </c>
+    </row>
+    <row r="16" ht="210" spans="1:6">
       <c r="B16" s="5" t="s">
-        <v>370</v>
+        <v>374</v>
       </c>
       <c r="C16" s="4"/>
       <c r="D16" t="s">
-        <v>372</v>
-      </c>
-      <c r="E16" s="18" t="s">
-        <v>413</v>
-      </c>
-    </row>
-    <row r="17" ht="43.5" spans="2:6">
+        <v>376</v>
+      </c>
+      <c r="E16" s="19" t="s">
+        <v>417</v>
+      </c>
+    </row>
+    <row r="17" ht="45" spans="2:6">
       <c r="B17" s="5" t="s">
-        <v>414</v>
+        <v>418</v>
       </c>
       <c r="C17" s="4" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="D17" s="4" t="s">
-        <v>415</v>
+        <v>419</v>
       </c>
     </row>
     <row r="18" spans="2:6">
       <c r="B18" t="s">
-        <v>374</v>
+        <v>378</v>
       </c>
       <c r="D18" t="s">
-        <v>375</v>
-      </c>
-      <c r="E18" s="8" t="s">
-        <v>426</v>
-      </c>
-      <c r="F18" s="19" t="s">
-        <v>376</v>
-      </c>
-    </row>
-    <row r="19" ht="159.5" spans="2:6">
+        <v>379</v>
+      </c>
+      <c r="E18" s="9" t="s">
+        <v>431</v>
+      </c>
+      <c r="F18" s="20" t="s">
+        <v>380</v>
+      </c>
+    </row>
+    <row r="19" ht="165" spans="2:6">
       <c r="B19" t="s">
-        <v>427</v>
+        <v>432</v>
       </c>
       <c r="D19" s="4" t="s">
-        <v>428</v>
+        <v>433</v>
       </c>
       <c r="E19" t="s">
-        <v>429</v>
+        <v>434</v>
       </c>
     </row>
     <row r="20" spans="2:6">
       <c r="B20" s="4" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="C20" s="4" t="s">
-        <v>193</v>
-      </c>
-      <c r="D20" s="14" t="s">
-        <v>416</v>
+        <v>194</v>
+      </c>
+      <c r="D20" s="15" t="s">
+        <v>420</v>
       </c>
     </row>
     <row r="21" ht="46" customHeight="1" spans="2:6">
       <c r="B21" s="4" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="C21" s="4" t="s">
-        <v>378</v>
-      </c>
-      <c r="D21" s="14"/>
+        <v>382</v>
+      </c>
+      <c r="D21" s="15"/>
     </row>
   </sheetData>
   <mergeCells count="2">

</xml_diff>